<commit_message>
intro and template narratives to excel template
</commit_message>
<xml_diff>
--- a/Template_Build_survival_curve_hazard_ratio_20260420_DZ.xlsx
+++ b/Template_Build_survival_curve_hazard_ratio_20260420_DZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xinzhao/DS_Projects/build-survival-curve-hazardratio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE7429CE-72CD-C34A-A318-5887C8F8F914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{361676CD-7CC7-664E-81D1-9C4B6074D66D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="600" windowWidth="37220" windowHeight="21000" xr2:uid="{120A936B-BDCD-7149-9B97-5E03885B164C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>Hazard ratio</t>
   </si>
@@ -144,6 +144,9 @@
 Base survival proportion → hazard → apply hazard ratio to derive target hazard → target survival proportion
 The equations underlying this workflow are implemented directly through Excel formulas embedded in the relevant parameter cells. The method assumes that the hazard remains constant within each age interval.</t>
   </si>
+  <si>
+    <t>The template comprises two components: input and output. In the input section, users can replace the example data in the table and hazard ratio table with their own data. Users can automatically obtain estimated target survival and mortality proportions at each age, in tabular and graphical formats.</t>
+  </si>
 </sst>
 </file>
 
@@ -152,7 +155,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -252,6 +255,18 @@
     <font>
       <sz val="15"/>
       <name val="Corbel"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1" tint="0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1" tint="0.34998626667073579"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -401,7 +416,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -494,9 +509,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="10" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -537,14 +549,20 @@
     <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1001,7 +1019,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Template!$C$27:$C$76</c:f>
+              <c:f>Template!$C$29:$C$78</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="50"/>
@@ -1160,7 +1178,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Template!$D$27:$D$76</c:f>
+              <c:f>Template!$D$29:$D$78</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="50"/>
@@ -1347,7 +1365,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Template!$O$27:$O$76</c:f>
+              <c:f>Template!$O$29:$O$78</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="50"/>
@@ -1506,7 +1524,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Template!$S$27:$S$76</c:f>
+              <c:f>Template!$S$29:$S$78</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="50"/>
@@ -2559,13 +2577,13 @@
     <xdr:from>
       <xdr:col>23</xdr:col>
       <xdr:colOff>56568</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>336846</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>33</xdr:col>
       <xdr:colOff>278509</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>101599</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2686,8 +2704,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3A341F5E-4E05-F048-996B-0F1926864DB8}" name="Table3" displayName="Table3" ref="G26:G27" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
-  <autoFilter ref="G26:G27" xr:uid="{3A341F5E-4E05-F048-996B-0F1926864DB8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3A341F5E-4E05-F048-996B-0F1926864DB8}" name="Table3" displayName="Table3" ref="G28:G29" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+  <autoFilter ref="G28:G29" xr:uid="{3A341F5E-4E05-F048-996B-0F1926864DB8}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{2B5CA90E-78A3-D647-B3E0-96A99414C2FE}" name="Hazard ratio" dataDxfId="13"/>
   </tableColumns>
@@ -2696,24 +2714,24 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7EB2E43A-16B5-4844-A683-8233B4340B9D}" name="Table1" displayName="Table1" ref="O26:T77" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11" dataCellStyle="Percent">
-  <autoFilter ref="O26:T77" xr:uid="{7EB2E43A-16B5-4844-A683-8233B4340B9D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7EB2E43A-16B5-4844-A683-8233B4340B9D}" name="Table1" displayName="Table1" ref="O28:T79" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11" dataCellStyle="Percent">
+  <autoFilter ref="O28:T79" xr:uid="{7EB2E43A-16B5-4844-A683-8233B4340B9D}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{24A47CF1-FBEC-8645-A58F-56A0E90B818A}" name="Age (year)" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{E29AE380-310C-6C46-B75E-D7BD3E83E1E7}" name="Survival, base" dataDxfId="9">
-      <calculatedColumnFormula>D27</calculatedColumnFormula>
+      <calculatedColumnFormula>D29</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{949A1760-5DDB-934C-9176-C40C2C47A156}" name="Hazard, base" dataDxfId="8" dataCellStyle="Percent">
-      <calculatedColumnFormula>IFERROR(-LN(P28/P27),"n/a")</calculatedColumnFormula>
+      <calculatedColumnFormula>IFERROR(-LN(P30/P29),"n/a")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{CBEDCA30-B180-6C43-B47E-4FC0153B12C9}" name="Hazard, target" dataDxfId="7">
-      <calculatedColumnFormula>IFERROR(Q27*$G$27,"n/a")</calculatedColumnFormula>
+      <calculatedColumnFormula>IFERROR(Q29*$G$29,"n/a")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{5DBE99A3-4E8F-784B-AB05-FFD71CB9D0E7}" name="Survival, target" dataDxfId="6" dataCellStyle="Percent">
-      <calculatedColumnFormula>IFERROR(S26*EXP(-R27),"n/a")</calculatedColumnFormula>
+      <calculatedColumnFormula>IFERROR(S28*EXP(-R29),"n/a")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{0DEFF837-9E36-CC46-9843-1B14030B9919}" name="CumEvent, target" dataDxfId="5" dataCellStyle="Percent">
-      <calculatedColumnFormula>IFERROR(1-S27, "n/a")</calculatedColumnFormula>
+      <calculatedColumnFormula>IFERROR(1-S29, "n/a")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2721,8 +2739,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{889A1322-1FFD-5C4E-A3E9-68606B33A535}" name="Table2" displayName="Table2" ref="C26:D77" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3" tableBorderDxfId="2">
-  <autoFilter ref="C26:D77" xr:uid="{889A1322-1FFD-5C4E-A3E9-68606B33A535}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{889A1322-1FFD-5C4E-A3E9-68606B33A535}" name="Table2" displayName="Table2" ref="C28:D79" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3" tableBorderDxfId="2">
+  <autoFilter ref="C28:D79" xr:uid="{889A1322-1FFD-5C4E-A3E9-68606B33A535}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{2A993501-0921-3A4F-93A2-743BC170CD7D}" name="Age (year)" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{88328291-4A16-9344-8559-DB82D115BB87}" name="Survival, base" dataDxfId="0"/>
@@ -3048,7 +3066,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A3DAE5-C576-0C46-AA24-CA8BC1EAE5FA}">
-  <dimension ref="A1:AU151"/>
+  <dimension ref="A1:AU155"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="16" zeroHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="10.83203125" style="2" customWidth="1"/>
@@ -3064,10 +3082,10 @@
     <col min="48" max="16384" width="10.83203125" style="2" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:47" s="8" customFormat="1" ht="108" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:47" s="8" customFormat="1" ht="140" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
-      <c r="K1" s="46" t="s">
+      <c r="K1" s="45" t="s">
         <v>16</v>
       </c>
       <c r="AT1"/>
@@ -3085,7 +3103,7 @@
       <c r="AP2"/>
       <c r="AQ2"/>
       <c r="AR2"/>
-      <c r="AT2" s="40"/>
+      <c r="AT2" s="39"/>
     </row>
     <row r="3" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AH3"/>
@@ -3099,7 +3117,7 @@
       <c r="AP3"/>
       <c r="AQ3"/>
       <c r="AR3"/>
-      <c r="AT3" s="40"/>
+      <c r="AT3" s="39"/>
     </row>
     <row r="4" spans="2:47" ht="24" x14ac:dyDescent="0.2">
       <c r="C4" s="28"/>
@@ -3133,28 +3151,28 @@
       <c r="AP4"/>
       <c r="AQ4"/>
       <c r="AR4"/>
-      <c r="AT4" s="40"/>
+      <c r="AT4" s="39"/>
     </row>
     <row r="5" spans="2:47" ht="28" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="31"/>
-      <c r="C5" s="32" t="s">
+      <c r="B5" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="34"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="34"/>
-      <c r="N5" s="34"/>
-      <c r="O5" s="34"/>
-      <c r="P5" s="34"/>
-      <c r="Q5" s="34"/>
-      <c r="R5" s="34"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
+      <c r="K5" s="33"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="33"/>
+      <c r="N5" s="33"/>
+      <c r="O5" s="33"/>
+      <c r="P5" s="33"/>
+      <c r="Q5" s="33"/>
+      <c r="R5" s="33"/>
       <c r="S5" s="30"/>
       <c r="T5" s="30"/>
       <c r="U5" s="30"/>
@@ -3181,26 +3199,26 @@
       <c r="AP5"/>
       <c r="AQ5"/>
       <c r="AR5"/>
-      <c r="AT5" s="40"/>
+      <c r="AT5" s="39"/>
     </row>
     <row r="6" spans="2:47" ht="28" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B6" s="31"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="35"/>
-      <c r="I6" s="35"/>
-      <c r="J6" s="35"/>
-      <c r="K6" s="35"/>
-      <c r="L6" s="35"/>
-      <c r="M6" s="35"/>
-      <c r="N6" s="35"/>
-      <c r="O6" s="35"/>
-      <c r="P6" s="35"/>
-      <c r="Q6" s="35"/>
-      <c r="R6" s="35"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="34"/>
+      <c r="L6" s="34"/>
+      <c r="M6" s="34"/>
+      <c r="N6" s="34"/>
+      <c r="O6" s="34"/>
+      <c r="P6" s="34"/>
+      <c r="Q6" s="34"/>
+      <c r="R6" s="34"/>
       <c r="S6" s="28"/>
       <c r="T6" s="28"/>
       <c r="U6" s="28"/>
@@ -3216,26 +3234,26 @@
       <c r="AP6"/>
       <c r="AQ6"/>
       <c r="AR6"/>
-      <c r="AT6" s="40"/>
+      <c r="AT6" s="39"/>
     </row>
     <row r="7" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B7" s="31"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="35"/>
-      <c r="K7" s="35"/>
-      <c r="L7" s="35"/>
-      <c r="M7" s="35"/>
-      <c r="N7" s="35"/>
-      <c r="O7" s="35"/>
-      <c r="P7" s="35"/>
-      <c r="Q7" s="35"/>
-      <c r="R7" s="35"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
+      <c r="K7" s="34"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="34"/>
+      <c r="N7" s="34"/>
+      <c r="O7" s="34"/>
+      <c r="P7" s="34"/>
+      <c r="Q7" s="34"/>
+      <c r="R7" s="34"/>
       <c r="S7" s="28"/>
       <c r="T7" s="28"/>
       <c r="U7" s="28"/>
@@ -3251,43 +3269,43 @@
       <c r="AP7"/>
       <c r="AQ7"/>
       <c r="AR7"/>
-      <c r="AT7" s="40"/>
+      <c r="AT7" s="39"/>
     </row>
     <row r="8" spans="2:47" ht="257" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="31"/>
-      <c r="C8" s="47" t="s">
+      <c r="C8" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="47"/>
-      <c r="E8" s="47"/>
-      <c r="F8" s="47"/>
-      <c r="G8" s="47"/>
-      <c r="H8" s="47"/>
-      <c r="I8" s="47"/>
-      <c r="J8" s="47"/>
-      <c r="K8" s="47"/>
-      <c r="L8" s="47"/>
-      <c r="M8" s="47"/>
-      <c r="N8" s="47"/>
-      <c r="O8" s="47"/>
-      <c r="P8" s="47"/>
-      <c r="Q8" s="47"/>
-      <c r="R8" s="47"/>
-      <c r="S8" s="47"/>
-      <c r="T8" s="47"/>
-      <c r="U8" s="48"/>
-      <c r="V8" s="48"/>
-      <c r="W8" s="48"/>
-      <c r="X8" s="48"/>
-      <c r="Y8" s="48"/>
-      <c r="Z8" s="48"/>
-      <c r="AA8" s="48"/>
-      <c r="AB8" s="48"/>
-      <c r="AC8" s="48"/>
-      <c r="AD8" s="48"/>
-      <c r="AE8" s="48"/>
-      <c r="AF8" s="48"/>
-      <c r="AG8" s="49"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="49"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="49"/>
+      <c r="H8" s="49"/>
+      <c r="I8" s="49"/>
+      <c r="J8" s="49"/>
+      <c r="K8" s="49"/>
+      <c r="L8" s="49"/>
+      <c r="M8" s="49"/>
+      <c r="N8" s="49"/>
+      <c r="O8" s="49"/>
+      <c r="P8" s="49"/>
+      <c r="Q8" s="49"/>
+      <c r="R8" s="49"/>
+      <c r="S8" s="49"/>
+      <c r="T8" s="49"/>
+      <c r="U8" s="46"/>
+      <c r="V8" s="46"/>
+      <c r="W8" s="46"/>
+      <c r="X8" s="46"/>
+      <c r="Y8" s="46"/>
+      <c r="Z8" s="46"/>
+      <c r="AA8" s="46"/>
+      <c r="AB8" s="46"/>
+      <c r="AC8" s="46"/>
+      <c r="AD8" s="46"/>
+      <c r="AE8" s="46"/>
+      <c r="AF8" s="46"/>
+      <c r="AG8" s="47"/>
       <c r="AH8"/>
       <c r="AI8"/>
       <c r="AJ8"/>
@@ -3299,28 +3317,28 @@
       <c r="AP8"/>
       <c r="AQ8"/>
       <c r="AR8"/>
-      <c r="AT8" s="40"/>
+      <c r="AT8" s="39"/>
     </row>
     <row r="9" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B9" s="31"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="35"/>
-      <c r="L9" s="35"/>
-      <c r="M9" s="35"/>
-      <c r="N9" s="35"/>
-      <c r="O9" s="35"/>
-      <c r="P9" s="35"/>
-      <c r="Q9" s="35"/>
-      <c r="R9" s="35"/>
-      <c r="S9" s="28"/>
-      <c r="T9" s="28"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="49"/>
+      <c r="K9" s="49"/>
+      <c r="L9" s="49"/>
+      <c r="M9" s="49"/>
+      <c r="N9" s="49"/>
+      <c r="O9" s="49"/>
+      <c r="P9" s="49"/>
+      <c r="Q9" s="49"/>
+      <c r="R9" s="49"/>
+      <c r="S9" s="49"/>
+      <c r="T9" s="49"/>
       <c r="U9" s="28"/>
       <c r="V9" s="28"/>
       <c r="AH9"/>
@@ -3334,28 +3352,28 @@
       <c r="AP9"/>
       <c r="AQ9"/>
       <c r="AR9"/>
-      <c r="AT9" s="40"/>
+      <c r="AT9" s="39"/>
     </row>
     <row r="10" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B10" s="31"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="35"/>
-      <c r="L10" s="35"/>
-      <c r="M10" s="35"/>
-      <c r="N10" s="35"/>
-      <c r="O10" s="35"/>
-      <c r="P10" s="35"/>
-      <c r="Q10" s="35"/>
-      <c r="R10" s="35"/>
-      <c r="S10" s="28"/>
-      <c r="T10" s="28"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+      <c r="M10" s="49"/>
+      <c r="N10" s="49"/>
+      <c r="O10" s="49"/>
+      <c r="P10" s="49"/>
+      <c r="Q10" s="49"/>
+      <c r="R10" s="49"/>
+      <c r="S10" s="49"/>
+      <c r="T10" s="49"/>
       <c r="U10" s="28"/>
       <c r="V10" s="28"/>
       <c r="AH10"/>
@@ -3369,26 +3387,26 @@
       <c r="AP10"/>
       <c r="AQ10"/>
       <c r="AR10"/>
-      <c r="AT10" s="40"/>
+      <c r="AT10" s="39"/>
     </row>
     <row r="11" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B11" s="31"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
-      <c r="J11" s="35"/>
-      <c r="K11" s="35"/>
-      <c r="L11" s="35"/>
-      <c r="M11" s="35"/>
-      <c r="N11" s="35"/>
-      <c r="O11" s="35"/>
-      <c r="P11" s="35"/>
-      <c r="Q11" s="35"/>
-      <c r="R11" s="35"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="34"/>
+      <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
+      <c r="M11" s="34"/>
+      <c r="N11" s="34"/>
+      <c r="O11" s="34"/>
+      <c r="P11" s="34"/>
+      <c r="Q11" s="34"/>
+      <c r="R11" s="34"/>
       <c r="S11" s="28"/>
       <c r="T11" s="28"/>
       <c r="U11" s="28"/>
@@ -3404,26 +3422,26 @@
       <c r="AP11"/>
       <c r="AQ11"/>
       <c r="AR11"/>
-      <c r="AT11" s="40"/>
+      <c r="AT11" s="39"/>
     </row>
     <row r="12" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B12" s="31"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35"/>
-      <c r="K12" s="35"/>
-      <c r="L12" s="35"/>
-      <c r="M12" s="35"/>
-      <c r="N12" s="35"/>
-      <c r="O12" s="35"/>
-      <c r="P12" s="35"/>
-      <c r="Q12" s="35"/>
-      <c r="R12" s="35"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="34"/>
+      <c r="J12" s="34"/>
+      <c r="K12" s="34"/>
+      <c r="L12" s="34"/>
+      <c r="M12" s="34"/>
+      <c r="N12" s="34"/>
+      <c r="O12" s="34"/>
+      <c r="P12" s="34"/>
+      <c r="Q12" s="34"/>
+      <c r="R12" s="34"/>
       <c r="S12" s="28"/>
       <c r="T12" s="28"/>
       <c r="U12" s="28"/>
@@ -3439,15 +3457,13 @@
       <c r="AP12"/>
       <c r="AQ12"/>
       <c r="AR12"/>
-      <c r="AT12" s="40"/>
-    </row>
-    <row r="13" spans="2:47" ht="28" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AT12" s="39"/>
+    </row>
+    <row r="13" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B13" s="31"/>
-      <c r="C13" s="37" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" s="33"/>
-      <c r="E13" s="33"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
       <c r="F13" s="34"/>
       <c r="G13" s="34"/>
       <c r="H13" s="34"/>
@@ -3461,25 +3477,14 @@
       <c r="P13" s="34"/>
       <c r="Q13" s="34"/>
       <c r="R13" s="34"/>
-      <c r="S13" s="30"/>
-      <c r="T13" s="30"/>
-      <c r="U13" s="30"/>
-      <c r="V13" s="30"/>
-      <c r="W13" s="10"/>
-      <c r="X13" s="10"/>
-      <c r="Y13" s="10"/>
-      <c r="Z13" s="10"/>
-      <c r="AA13" s="10"/>
-      <c r="AB13" s="10"/>
-      <c r="AC13" s="10"/>
-      <c r="AD13" s="10"/>
-      <c r="AE13" s="10"/>
-      <c r="AF13" s="10"/>
-      <c r="AG13" s="10"/>
-      <c r="AH13" s="12"/>
-      <c r="AI13" s="12"/>
-      <c r="AJ13" s="12"/>
-      <c r="AK13" s="12"/>
+      <c r="S13" s="28"/>
+      <c r="T13" s="28"/>
+      <c r="U13" s="28"/>
+      <c r="V13" s="28"/>
+      <c r="AH13"/>
+      <c r="AI13"/>
+      <c r="AJ13"/>
+      <c r="AK13"/>
       <c r="AL13"/>
       <c r="AM13"/>
       <c r="AN13"/>
@@ -3487,26 +3492,26 @@
       <c r="AP13"/>
       <c r="AQ13"/>
       <c r="AR13"/>
-      <c r="AT13" s="40"/>
-    </row>
-    <row r="14" spans="2:47" ht="28" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="AT13" s="39"/>
+    </row>
+    <row r="14" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B14" s="31"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="35"/>
-      <c r="L14" s="35"/>
-      <c r="M14" s="35"/>
-      <c r="N14" s="35"/>
-      <c r="O14" s="35"/>
-      <c r="P14" s="35"/>
-      <c r="Q14" s="35"/>
-      <c r="R14" s="35"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
+      <c r="I14" s="34"/>
+      <c r="J14" s="34"/>
+      <c r="K14" s="34"/>
+      <c r="L14" s="34"/>
+      <c r="M14" s="34"/>
+      <c r="N14" s="34"/>
+      <c r="O14" s="34"/>
+      <c r="P14" s="34"/>
+      <c r="Q14" s="34"/>
+      <c r="R14" s="34"/>
       <c r="S14" s="28"/>
       <c r="T14" s="28"/>
       <c r="U14" s="28"/>
@@ -3522,26 +3527,26 @@
       <c r="AP14"/>
       <c r="AQ14"/>
       <c r="AR14"/>
-      <c r="AT14" s="40"/>
+      <c r="AT14" s="39"/>
     </row>
     <row r="15" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B15" s="31"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="35"/>
-      <c r="L15" s="35"/>
-      <c r="M15" s="35"/>
-      <c r="N15" s="35"/>
-      <c r="O15" s="35"/>
-      <c r="P15" s="35"/>
-      <c r="Q15" s="35"/>
-      <c r="R15" s="35"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="34"/>
+      <c r="J15" s="34"/>
+      <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
+      <c r="M15" s="34"/>
+      <c r="N15" s="34"/>
+      <c r="O15" s="34"/>
+      <c r="P15" s="34"/>
+      <c r="Q15" s="34"/>
+      <c r="R15" s="34"/>
       <c r="S15" s="28"/>
       <c r="T15" s="28"/>
       <c r="U15" s="28"/>
@@ -3557,26 +3562,26 @@
       <c r="AP15"/>
       <c r="AQ15"/>
       <c r="AR15"/>
-      <c r="AT15" s="40"/>
+      <c r="AT15" s="39"/>
     </row>
     <row r="16" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B16" s="31"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="36"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="35"/>
-      <c r="L16" s="35"/>
-      <c r="M16" s="35"/>
-      <c r="N16" s="35"/>
-      <c r="O16" s="35"/>
-      <c r="P16" s="35"/>
-      <c r="Q16" s="35"/>
-      <c r="R16" s="35"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+      <c r="I16" s="34"/>
+      <c r="J16" s="34"/>
+      <c r="K16" s="34"/>
+      <c r="L16" s="34"/>
+      <c r="M16" s="34"/>
+      <c r="N16" s="34"/>
+      <c r="O16" s="34"/>
+      <c r="P16" s="34"/>
+      <c r="Q16" s="34"/>
+      <c r="R16" s="34"/>
       <c r="S16" s="28"/>
       <c r="T16" s="28"/>
       <c r="U16" s="28"/>
@@ -3592,34 +3597,47 @@
       <c r="AP16"/>
       <c r="AQ16"/>
       <c r="AR16"/>
-      <c r="AT16" s="40"/>
-    </row>
-    <row r="17" spans="2:46" ht="27" x14ac:dyDescent="0.2">
-      <c r="B17" s="31"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="35"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
-      <c r="J17" s="35"/>
-      <c r="K17" s="35"/>
-      <c r="L17" s="35"/>
-      <c r="M17" s="35"/>
-      <c r="N17" s="35"/>
-      <c r="O17" s="35"/>
-      <c r="P17" s="35"/>
-      <c r="Q17" s="35"/>
-      <c r="R17" s="35"/>
-      <c r="S17" s="28"/>
-      <c r="T17" s="28"/>
-      <c r="U17" s="28"/>
-      <c r="V17" s="28"/>
-      <c r="AH17"/>
-      <c r="AI17"/>
-      <c r="AJ17"/>
-      <c r="AK17"/>
+      <c r="AT16" s="39"/>
+    </row>
+    <row r="17" spans="2:46" ht="28" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="36" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
+      <c r="J17" s="33"/>
+      <c r="K17" s="33"/>
+      <c r="L17" s="33"/>
+      <c r="M17" s="33"/>
+      <c r="N17" s="33"/>
+      <c r="O17" s="33"/>
+      <c r="P17" s="33"/>
+      <c r="Q17" s="33"/>
+      <c r="R17" s="33"/>
+      <c r="S17" s="30"/>
+      <c r="T17" s="30"/>
+      <c r="U17" s="30"/>
+      <c r="V17" s="30"/>
+      <c r="W17" s="10"/>
+      <c r="X17" s="10"/>
+      <c r="Y17" s="10"/>
+      <c r="Z17" s="10"/>
+      <c r="AA17" s="10"/>
+      <c r="AB17" s="10"/>
+      <c r="AC17" s="10"/>
+      <c r="AD17" s="10"/>
+      <c r="AE17" s="10"/>
+      <c r="AF17" s="10"/>
+      <c r="AG17" s="10"/>
+      <c r="AH17" s="12"/>
+      <c r="AI17" s="12"/>
+      <c r="AJ17" s="12"/>
+      <c r="AK17" s="12"/>
       <c r="AL17"/>
       <c r="AM17"/>
       <c r="AN17"/>
@@ -3627,47 +3645,32 @@
       <c r="AP17"/>
       <c r="AQ17"/>
       <c r="AR17"/>
-      <c r="AT17" s="40"/>
-    </row>
-    <row r="18" spans="2:46" ht="28" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AT17" s="39"/>
+    </row>
+    <row r="18" spans="2:46" ht="28" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B18" s="31"/>
-      <c r="C18" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
       <c r="F18" s="34"/>
       <c r="G18" s="34"/>
       <c r="H18" s="34"/>
       <c r="I18" s="34"/>
       <c r="J18" s="34"/>
-      <c r="K18" s="35"/>
-      <c r="L18" s="35"/>
-      <c r="M18" s="35"/>
-      <c r="N18" s="35"/>
-      <c r="O18" s="37" t="s">
-        <v>15</v>
-      </c>
+      <c r="K18" s="34"/>
+      <c r="L18" s="34"/>
+      <c r="M18" s="34"/>
+      <c r="N18" s="34"/>
+      <c r="O18" s="34"/>
       <c r="P18" s="34"/>
       <c r="Q18" s="34"/>
       <c r="R18" s="34"/>
-      <c r="S18" s="30"/>
-      <c r="T18" s="30"/>
-      <c r="U18" s="30"/>
-      <c r="V18" s="30"/>
-      <c r="W18" s="10"/>
-      <c r="X18" s="10"/>
-      <c r="Y18" s="10"/>
-      <c r="Z18" s="10"/>
-      <c r="AA18" s="10"/>
-      <c r="AB18" s="10"/>
-      <c r="AC18" s="10"/>
-      <c r="AD18" s="10"/>
-      <c r="AE18" s="10"/>
-      <c r="AF18" s="10"/>
-      <c r="AG18" s="10"/>
-      <c r="AH18" s="10"/>
-      <c r="AI18" s="10"/>
+      <c r="S18" s="28"/>
+      <c r="T18" s="28"/>
+      <c r="U18" s="28"/>
+      <c r="V18" s="28"/>
+      <c r="AH18"/>
+      <c r="AI18"/>
       <c r="AJ18"/>
       <c r="AK18"/>
       <c r="AL18"/>
@@ -3677,9 +3680,34 @@
       <c r="AP18"/>
       <c r="AQ18"/>
       <c r="AR18"/>
-      <c r="AT18" s="40"/>
-    </row>
-    <row r="19" spans="2:46" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="AT18" s="39"/>
+    </row>
+    <row r="19" spans="2:46" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="31"/>
+      <c r="C19" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="50"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="N19" s="50"/>
+      <c r="O19" s="50"/>
+      <c r="P19" s="50"/>
+      <c r="Q19" s="50"/>
+      <c r="R19" s="50"/>
+      <c r="S19" s="50"/>
+      <c r="T19" s="50"/>
+      <c r="U19" s="28"/>
+      <c r="V19" s="28"/>
+      <c r="AH19"/>
+      <c r="AI19"/>
       <c r="AJ19"/>
       <c r="AK19"/>
       <c r="AL19"/>
@@ -3689,9 +3717,32 @@
       <c r="AP19"/>
       <c r="AQ19"/>
       <c r="AR19"/>
-      <c r="AT19" s="40"/>
-    </row>
-    <row r="20" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="AT19" s="39"/>
+    </row>
+    <row r="20" spans="2:46" ht="27" x14ac:dyDescent="0.2">
+      <c r="B20" s="31"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
+      <c r="I20" s="34"/>
+      <c r="J20" s="34"/>
+      <c r="K20" s="34"/>
+      <c r="L20" s="34"/>
+      <c r="M20" s="34"/>
+      <c r="N20" s="34"/>
+      <c r="O20" s="34"/>
+      <c r="P20" s="34"/>
+      <c r="Q20" s="34"/>
+      <c r="R20" s="34"/>
+      <c r="S20" s="28"/>
+      <c r="T20" s="28"/>
+      <c r="U20" s="28"/>
+      <c r="V20" s="28"/>
+      <c r="AH20"/>
+      <c r="AI20"/>
       <c r="AJ20"/>
       <c r="AK20"/>
       <c r="AL20"/>
@@ -3701,9 +3752,32 @@
       <c r="AP20"/>
       <c r="AQ20"/>
       <c r="AR20"/>
-      <c r="AT20" s="40"/>
-    </row>
-    <row r="21" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="AT20" s="39"/>
+    </row>
+    <row r="21" spans="2:46" ht="27" x14ac:dyDescent="0.2">
+      <c r="B21" s="31"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="34"/>
+      <c r="J21" s="34"/>
+      <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
+      <c r="M21" s="34"/>
+      <c r="N21" s="34"/>
+      <c r="O21" s="34"/>
+      <c r="P21" s="34"/>
+      <c r="Q21" s="34"/>
+      <c r="R21" s="34"/>
+      <c r="S21" s="28"/>
+      <c r="T21" s="28"/>
+      <c r="U21" s="28"/>
+      <c r="V21" s="28"/>
+      <c r="AH21"/>
+      <c r="AI21"/>
       <c r="AJ21"/>
       <c r="AK21"/>
       <c r="AL21"/>
@@ -3713,9 +3787,47 @@
       <c r="AP21"/>
       <c r="AQ21"/>
       <c r="AR21"/>
-      <c r="AT21" s="40"/>
-    </row>
-    <row r="22" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="AT21" s="39"/>
+    </row>
+    <row r="22" spans="2:46" ht="28" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="31"/>
+      <c r="C22" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="34"/>
+      <c r="L22" s="34"/>
+      <c r="M22" s="34"/>
+      <c r="N22" s="34"/>
+      <c r="O22" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="P22" s="33"/>
+      <c r="Q22" s="33"/>
+      <c r="R22" s="33"/>
+      <c r="S22" s="30"/>
+      <c r="T22" s="30"/>
+      <c r="U22" s="30"/>
+      <c r="V22" s="30"/>
+      <c r="W22" s="10"/>
+      <c r="X22" s="10"/>
+      <c r="Y22" s="10"/>
+      <c r="Z22" s="10"/>
+      <c r="AA22" s="10"/>
+      <c r="AB22" s="10"/>
+      <c r="AC22" s="10"/>
+      <c r="AD22" s="10"/>
+      <c r="AE22" s="10"/>
+      <c r="AF22" s="10"/>
+      <c r="AG22" s="10"/>
+      <c r="AH22" s="10"/>
+      <c r="AI22" s="10"/>
       <c r="AJ22"/>
       <c r="AK22"/>
       <c r="AL22"/>
@@ -3725,9 +3837,9 @@
       <c r="AP22"/>
       <c r="AQ22"/>
       <c r="AR22"/>
-      <c r="AT22" s="40"/>
-    </row>
-    <row r="23" spans="2:46" x14ac:dyDescent="0.2">
+      <c r="AT22" s="39"/>
+    </row>
+    <row r="23" spans="2:46" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="AJ23"/>
       <c r="AK23"/>
       <c r="AL23"/>
@@ -3737,36 +3849,9 @@
       <c r="AP23"/>
       <c r="AQ23"/>
       <c r="AR23"/>
-      <c r="AT23" s="40"/>
-    </row>
-    <row r="24" spans="2:46" s="4" customFormat="1" ht="24" x14ac:dyDescent="0.2">
-      <c r="C24" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="6"/>
-      <c r="E24" s="11"/>
-      <c r="G24" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="O24" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="P24" s="5"/>
-      <c r="Q24" s="5"/>
-      <c r="R24" s="5"/>
-      <c r="X24" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="Y24" s="5"/>
-      <c r="Z24" s="5"/>
-      <c r="AA24" s="5"/>
-      <c r="AB24" s="5"/>
-      <c r="AC24" s="5"/>
-      <c r="AD24" s="5"/>
-      <c r="AE24" s="5"/>
-      <c r="AF24" s="5"/>
-      <c r="AG24" s="5"/>
-      <c r="AH24" s="5"/>
+      <c r="AT23" s="39"/>
+    </row>
+    <row r="24" spans="2:46" x14ac:dyDescent="0.2">
       <c r="AJ24"/>
       <c r="AK24"/>
       <c r="AL24"/>
@@ -3776,8 +3861,7 @@
       <c r="AP24"/>
       <c r="AQ24"/>
       <c r="AR24"/>
-      <c r="AS24"/>
-      <c r="AT24" s="40"/>
+      <c r="AT24" s="39"/>
     </row>
     <row r="25" spans="2:46" x14ac:dyDescent="0.2">
       <c r="AJ25"/>
@@ -3789,37 +3873,36 @@
       <c r="AP25"/>
       <c r="AQ25"/>
       <c r="AR25"/>
-      <c r="AT25" s="40"/>
-    </row>
-    <row r="26" spans="2:46" s="1" customFormat="1" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="C26" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="E26"/>
-      <c r="G26" s="1" t="s">
+      <c r="AT25" s="39"/>
+    </row>
+    <row r="26" spans="2:46" s="4" customFormat="1" ht="24" x14ac:dyDescent="0.2">
+      <c r="C26" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="6"/>
+      <c r="E26" s="11"/>
+      <c r="G26" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="O26" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="P26" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q26" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="R26" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="S26" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="T26" s="13" t="s">
-        <v>13</v>
-      </c>
+      <c r="O26" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="P26" s="5"/>
+      <c r="Q26" s="5"/>
+      <c r="R26" s="5"/>
+      <c r="X26" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y26" s="5"/>
+      <c r="Z26" s="5"/>
+      <c r="AA26" s="5"/>
+      <c r="AB26" s="5"/>
+      <c r="AC26" s="5"/>
+      <c r="AD26" s="5"/>
+      <c r="AE26" s="5"/>
+      <c r="AF26" s="5"/>
+      <c r="AG26" s="5"/>
+      <c r="AH26" s="5"/>
       <c r="AJ26"/>
       <c r="AK26"/>
       <c r="AL26"/>
@@ -3830,42 +3913,9 @@
       <c r="AQ26"/>
       <c r="AR26"/>
       <c r="AS26"/>
-      <c r="AT26" s="40"/>
+      <c r="AT26" s="39"/>
     </row>
     <row r="27" spans="2:46" x14ac:dyDescent="0.2">
-      <c r="C27" s="19">
-        <v>0</v>
-      </c>
-      <c r="D27" s="22">
-        <v>1</v>
-      </c>
-      <c r="E27"/>
-      <c r="G27" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="O27" s="24">
-        <v>0</v>
-      </c>
-      <c r="P27" s="15">
-        <f>D27</f>
-        <v>1</v>
-      </c>
-      <c r="Q27" s="16">
-        <f>IFERROR(-LN(P28/P27),"n/a")</f>
-        <v>0</v>
-      </c>
-      <c r="R27" s="17">
-        <f>IFERROR(Q27*$G$27,"n/a")</f>
-        <v>0</v>
-      </c>
-      <c r="S27" s="18">
-        <f>Template!$P27</f>
-        <v>1</v>
-      </c>
-      <c r="T27" s="18">
-        <f>IFERROR(1-S27, "n/a")</f>
-        <v>0</v>
-      </c>
       <c r="AJ27"/>
       <c r="AK27"/>
       <c r="AL27"/>
@@ -3875,38 +3925,36 @@
       <c r="AP27"/>
       <c r="AQ27"/>
       <c r="AR27"/>
-      <c r="AT27" s="40"/>
-    </row>
-    <row r="28" spans="2:46" x14ac:dyDescent="0.2">
-      <c r="C28" s="20">
-        <v>1</v>
-      </c>
-      <c r="D28" s="21">
-        <v>1</v>
+      <c r="AT27" s="39"/>
+    </row>
+    <row r="28" spans="2:46" s="1" customFormat="1" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C28" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>8</v>
       </c>
       <c r="E28"/>
-      <c r="O28" s="24">
-        <v>1</v>
-      </c>
-      <c r="P28" s="15">
-        <f t="shared" ref="P28:P77" si="0">D28</f>
-        <v>1</v>
-      </c>
-      <c r="Q28" s="16">
-        <f t="shared" ref="Q28:Q77" si="1">IFERROR(-LN(P29/P28),"n/a")</f>
+      <c r="G28" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="R28" s="17">
-        <f t="shared" ref="R28:R77" si="2">IFERROR(Q28*$G$27,"n/a")</f>
-        <v>0</v>
-      </c>
-      <c r="S28" s="18">
-        <f>IFERROR(S27*EXP(-R28),"n/a")</f>
-        <v>1</v>
-      </c>
-      <c r="T28" s="18">
-        <f t="shared" ref="T28:T77" si="3">IFERROR(1-S28, "n/a")</f>
-        <v>0</v>
+      <c r="O28" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="P28" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q28" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="R28" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="S28" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="T28" s="13" t="s">
+        <v>13</v>
       </c>
       <c r="AJ28"/>
       <c r="AK28"/>
@@ -3917,37 +3965,41 @@
       <c r="AP28"/>
       <c r="AQ28"/>
       <c r="AR28"/>
-      <c r="AT28" s="40"/>
+      <c r="AS28"/>
+      <c r="AT28" s="39"/>
     </row>
     <row r="29" spans="2:46" x14ac:dyDescent="0.2">
-      <c r="C29" s="20">
-        <v>2</v>
-      </c>
-      <c r="D29" s="21">
+      <c r="C29" s="19">
+        <v>0</v>
+      </c>
+      <c r="D29" s="22">
         <v>1</v>
       </c>
       <c r="E29"/>
+      <c r="G29" s="7">
+        <v>0.5</v>
+      </c>
       <c r="O29" s="24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P29" s="15">
-        <f t="shared" si="0"/>
+        <f>D29</f>
         <v>1</v>
       </c>
       <c r="Q29" s="16">
-        <f t="shared" si="1"/>
+        <f>IFERROR(-LN(P30/P29),"n/a")</f>
         <v>0</v>
       </c>
       <c r="R29" s="17">
-        <f t="shared" si="2"/>
+        <f>IFERROR(Q29*$G$29,"n/a")</f>
         <v>0</v>
       </c>
       <c r="S29" s="18">
-        <f t="shared" ref="S29:S77" si="4">IFERROR(S28*EXP(-R29),"n/a")</f>
+        <f>Template!$P29</f>
         <v>1</v>
       </c>
       <c r="T29" s="18">
-        <f t="shared" si="3"/>
+        <f>IFERROR(1-S29, "n/a")</f>
         <v>0</v>
       </c>
       <c r="AJ29"/>
@@ -3959,37 +4011,37 @@
       <c r="AP29"/>
       <c r="AQ29"/>
       <c r="AR29"/>
-      <c r="AT29" s="40"/>
+      <c r="AT29" s="39"/>
     </row>
     <row r="30" spans="2:46" x14ac:dyDescent="0.2">
       <c r="C30" s="20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" s="21">
         <v>1</v>
       </c>
       <c r="E30"/>
       <c r="O30" s="24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P30" s="15">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="P30:P79" si="0">D30</f>
         <v>1</v>
       </c>
       <c r="Q30" s="16">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="Q30:Q79" si="1">IFERROR(-LN(P31/P30),"n/a")</f>
         <v>0</v>
       </c>
       <c r="R30" s="17">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="R30:R79" si="2">IFERROR(Q30*$G$29,"n/a")</f>
         <v>0</v>
       </c>
       <c r="S30" s="18">
-        <f t="shared" si="4"/>
+        <f>IFERROR(S29*EXP(-R30),"n/a")</f>
         <v>1</v>
       </c>
       <c r="T30" s="18">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="T30:T79" si="3">IFERROR(1-S30, "n/a")</f>
         <v>0</v>
       </c>
       <c r="AJ30"/>
@@ -4001,18 +4053,18 @@
       <c r="AP30"/>
       <c r="AQ30"/>
       <c r="AR30"/>
-      <c r="AT30" s="40"/>
+      <c r="AT30" s="39"/>
     </row>
     <row r="31" spans="2:46" x14ac:dyDescent="0.2">
       <c r="C31" s="20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D31" s="21">
         <v>1</v>
       </c>
       <c r="E31"/>
       <c r="O31" s="24">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P31" s="15">
         <f t="shared" si="0"/>
@@ -4027,7 +4079,7 @@
         <v>0</v>
       </c>
       <c r="S31" s="18">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="S31:S79" si="4">IFERROR(S30*EXP(-R31),"n/a")</f>
         <v>1</v>
       </c>
       <c r="T31" s="18">
@@ -4043,18 +4095,18 @@
       <c r="AP31"/>
       <c r="AQ31"/>
       <c r="AR31"/>
-      <c r="AT31" s="40"/>
+      <c r="AT31" s="39"/>
     </row>
     <row r="32" spans="2:46" x14ac:dyDescent="0.2">
       <c r="C32" s="20">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D32" s="21">
         <v>1</v>
       </c>
       <c r="E32"/>
       <c r="O32" s="24">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P32" s="15">
         <f t="shared" si="0"/>
@@ -4062,19 +4114,19 @@
       </c>
       <c r="Q32" s="16">
         <f t="shared" si="1"/>
-        <v>8.913702984424896E-8</v>
+        <v>0</v>
       </c>
       <c r="R32" s="17">
         <f t="shared" si="2"/>
-        <v>4.456851492212448E-8</v>
+        <v>0</v>
       </c>
       <c r="S32" s="18">
         <f t="shared" si="4"/>
-        <v>0.99999995543148612</v>
+        <v>1</v>
       </c>
       <c r="T32" s="18">
         <f t="shared" si="3"/>
-        <v>4.4568513879461591E-8</v>
+        <v>0</v>
       </c>
       <c r="AJ32"/>
       <c r="AK32"/>
@@ -4085,38 +4137,38 @@
       <c r="AP32"/>
       <c r="AQ32"/>
       <c r="AR32"/>
-      <c r="AT32" s="40"/>
+      <c r="AT32" s="39"/>
     </row>
     <row r="33" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C33" s="20">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D33" s="21">
-        <v>0.99999991086297413</v>
+        <v>1</v>
       </c>
       <c r="E33"/>
       <c r="O33" s="24">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P33" s="15">
         <f t="shared" si="0"/>
-        <v>0.99999991086297413</v>
+        <v>1</v>
       </c>
       <c r="Q33" s="16">
         <f t="shared" si="1"/>
-        <v>9.038976005891162E-6</v>
+        <v>0</v>
       </c>
       <c r="R33" s="17">
         <f t="shared" si="2"/>
-        <v>4.519488002945581E-6</v>
+        <v>0</v>
       </c>
       <c r="S33" s="18">
         <f t="shared" si="4"/>
-        <v>0.99999543595389739</v>
+        <v>1</v>
       </c>
       <c r="T33" s="18">
         <f t="shared" si="3"/>
-        <v>4.5640461026064116E-6</v>
+        <v>0</v>
       </c>
       <c r="AJ33"/>
       <c r="AK33"/>
@@ -4127,38 +4179,38 @@
       <c r="AP33"/>
       <c r="AQ33"/>
       <c r="AR33"/>
-      <c r="AT33" s="40"/>
+      <c r="AT33" s="39"/>
     </row>
     <row r="34" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C34" s="20">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D34" s="21">
-        <v>0.99999087192862535</v>
+        <v>1</v>
       </c>
       <c r="E34"/>
       <c r="O34" s="24">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P34" s="15">
         <f t="shared" si="0"/>
-        <v>0.99999087192862535</v>
+        <v>1</v>
       </c>
       <c r="Q34" s="16">
         <f t="shared" si="1"/>
-        <v>1.3733291246540143E-4</v>
+        <v>8.913702984424896E-8</v>
       </c>
       <c r="R34" s="17">
         <f t="shared" si="2"/>
-        <v>6.8666456232700717E-5</v>
+        <v>4.456851492212448E-8</v>
       </c>
       <c r="S34" s="18">
         <f t="shared" si="4"/>
-        <v>0.99992677216853798</v>
+        <v>0.99999995543148612</v>
       </c>
       <c r="T34" s="18">
         <f t="shared" si="3"/>
-        <v>7.3227831462019388E-5</v>
+        <v>4.4568513879461591E-8</v>
       </c>
       <c r="AJ34"/>
       <c r="AK34"/>
@@ -4169,38 +4221,38 @@
       <c r="AP34"/>
       <c r="AQ34"/>
       <c r="AR34"/>
-      <c r="AT34" s="40"/>
+      <c r="AT34" s="39"/>
     </row>
     <row r="35" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C35" s="20">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D35" s="21">
-        <v>0.99985354969939122</v>
+        <v>0.99999991086297413</v>
       </c>
       <c r="E35"/>
       <c r="O35" s="24">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P35" s="15">
         <f t="shared" si="0"/>
-        <v>0.99985354969939122</v>
+        <v>0.99999991086297413</v>
       </c>
       <c r="Q35" s="16">
         <f t="shared" si="1"/>
-        <v>7.9999103752277493E-4</v>
+        <v>9.038976005891162E-6</v>
       </c>
       <c r="R35" s="17">
         <f t="shared" si="2"/>
-        <v>3.9999551876138747E-4</v>
+        <v>4.519488002945581E-6</v>
       </c>
       <c r="S35" s="18">
         <f t="shared" si="4"/>
-        <v>0.99952688592226602</v>
+        <v>0.99999543595389739</v>
       </c>
       <c r="T35" s="18">
         <f t="shared" si="3"/>
-        <v>4.7311407773398262E-4</v>
+        <v>4.5640461026064116E-6</v>
       </c>
       <c r="AJ35"/>
       <c r="AK35"/>
@@ -4211,38 +4263,38 @@
       <c r="AP35"/>
       <c r="AQ35"/>
       <c r="AR35"/>
-      <c r="AT35" s="40"/>
+      <c r="AT35" s="39"/>
     </row>
     <row r="36" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C36" s="20">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D36" s="21">
-        <v>0.99905399568146247</v>
+        <v>0.99999087192862535</v>
       </c>
       <c r="E36"/>
       <c r="O36" s="24">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P36" s="15">
         <f t="shared" si="0"/>
-        <v>0.99905399568146247</v>
+        <v>0.99999087192862535</v>
       </c>
       <c r="Q36" s="16">
         <f t="shared" si="1"/>
-        <v>2.6752916838612929E-3</v>
+        <v>1.3733291246540143E-4</v>
       </c>
       <c r="R36" s="17">
         <f t="shared" si="2"/>
-        <v>1.3376458419306464E-3</v>
+        <v>6.8666456232700717E-5</v>
       </c>
       <c r="S36" s="18">
         <f t="shared" si="4"/>
-        <v>0.99819076676575724</v>
+        <v>0.99992677216853798</v>
       </c>
       <c r="T36" s="18">
         <f t="shared" si="3"/>
-        <v>1.8092332342427575E-3</v>
+        <v>7.3227831462019388E-5</v>
       </c>
       <c r="AJ36"/>
       <c r="AK36"/>
@@ -4253,38 +4305,38 @@
       <c r="AP36"/>
       <c r="AQ36"/>
       <c r="AR36"/>
-      <c r="AT36" s="40"/>
+      <c r="AT36" s="39"/>
     </row>
     <row r="37" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C37" s="20">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D37" s="21">
-        <v>0.9963848068564104</v>
+        <v>0.99985354969939122</v>
       </c>
       <c r="E37"/>
       <c r="O37" s="24">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P37" s="15">
         <f t="shared" si="0"/>
-        <v>0.9963848068564104</v>
+        <v>0.99985354969939122</v>
       </c>
       <c r="Q37" s="16">
         <f t="shared" si="1"/>
-        <v>6.3200618049529022E-3</v>
+        <v>7.9999103752277493E-4</v>
       </c>
       <c r="R37" s="17">
         <f t="shared" si="2"/>
-        <v>3.1600309024764511E-3</v>
+        <v>3.9999551876138747E-4</v>
       </c>
       <c r="S37" s="18">
         <f t="shared" si="4"/>
-        <v>0.99504143171496962</v>
+        <v>0.99952688592226602</v>
       </c>
       <c r="T37" s="18">
         <f t="shared" si="3"/>
-        <v>4.9585682850303847E-3</v>
+        <v>4.7311407773398262E-4</v>
       </c>
       <c r="AJ37"/>
       <c r="AK37"/>
@@ -4295,38 +4347,38 @@
       <c r="AP37"/>
       <c r="AQ37"/>
       <c r="AR37"/>
-      <c r="AT37" s="40"/>
+      <c r="AT37" s="39"/>
     </row>
     <row r="38" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C38" s="20">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D38" s="21">
-        <v>0.99010745082937668</v>
+        <v>0.99905399568146247</v>
       </c>
       <c r="E38"/>
       <c r="O38" s="24">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="P38" s="15">
         <f t="shared" si="0"/>
-        <v>0.99010745082937668</v>
+        <v>0.99905399568146247</v>
       </c>
       <c r="Q38" s="16">
         <f t="shared" si="1"/>
-        <v>1.1865621989414932E-2</v>
+        <v>2.6752916838612929E-3</v>
       </c>
       <c r="R38" s="17">
         <f t="shared" si="2"/>
-        <v>5.9328109947074659E-3</v>
+        <v>1.3376458419306464E-3</v>
       </c>
       <c r="S38" s="18">
         <f t="shared" si="4"/>
-        <v>0.98915551624518983</v>
+        <v>0.99819076676575724</v>
       </c>
       <c r="T38" s="18">
         <f t="shared" si="3"/>
-        <v>1.0844483754810175E-2</v>
+        <v>1.8092332342427575E-3</v>
       </c>
       <c r="AJ38"/>
       <c r="AK38"/>
@@ -4337,38 +4389,38 @@
       <c r="AP38"/>
       <c r="AQ38"/>
       <c r="AR38"/>
-      <c r="AT38" s="40"/>
+      <c r="AT38" s="39"/>
     </row>
     <row r="39" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C39" s="20">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D39" s="21">
-        <v>0.97842863531828816</v>
+        <v>0.9963848068564104</v>
       </c>
       <c r="E39"/>
       <c r="O39" s="24">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="P39" s="15">
         <f t="shared" si="0"/>
-        <v>0.97842863531828816</v>
+        <v>0.9963848068564104</v>
       </c>
       <c r="Q39" s="16">
         <f t="shared" si="1"/>
-        <v>1.902355381396259E-2</v>
+        <v>6.3200618049529022E-3</v>
       </c>
       <c r="R39" s="17">
         <f t="shared" si="2"/>
-        <v>9.5117769069812952E-3</v>
+        <v>3.1600309024764511E-3</v>
       </c>
       <c r="S39" s="18">
         <f t="shared" si="4"/>
-        <v>0.97979149449115144</v>
+        <v>0.99504143171496962</v>
       </c>
       <c r="T39" s="18">
         <f t="shared" si="3"/>
-        <v>2.0208505508848562E-2</v>
+        <v>4.9585682850303847E-3</v>
       </c>
       <c r="AJ39"/>
       <c r="AK39"/>
@@ -4379,38 +4431,38 @@
       <c r="AP39"/>
       <c r="AQ39"/>
       <c r="AR39"/>
-      <c r="AT39" s="40"/>
+      <c r="AT39" s="39"/>
     </row>
     <row r="40" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C40" s="20">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D40" s="21">
-        <v>0.95999137267720414</v>
+        <v>0.99010745082937668</v>
       </c>
       <c r="E40"/>
       <c r="O40" s="24">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="P40" s="15">
         <f t="shared" si="0"/>
-        <v>0.95999137267720414</v>
+        <v>0.99010745082937668</v>
       </c>
       <c r="Q40" s="16">
         <f t="shared" si="1"/>
-        <v>2.7277023241003562E-2</v>
+        <v>1.1865621989414932E-2</v>
       </c>
       <c r="R40" s="17">
         <f t="shared" si="2"/>
-        <v>1.3638511620501781E-2</v>
+        <v>5.9328109947074659E-3</v>
       </c>
       <c r="S40" s="18">
         <f t="shared" si="4"/>
-        <v>0.9665193089643247</v>
+        <v>0.98915551624518983</v>
       </c>
       <c r="T40" s="18">
         <f t="shared" si="3"/>
-        <v>3.3480691035675303E-2</v>
+        <v>1.0844483754810175E-2</v>
       </c>
       <c r="AJ40"/>
       <c r="AK40"/>
@@ -4421,38 +4473,38 @@
       <c r="AP40"/>
       <c r="AQ40"/>
       <c r="AR40"/>
-      <c r="AT40" s="40"/>
+      <c r="AT40" s="39"/>
     </row>
     <row r="41" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C41" s="20">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D41" s="21">
-        <v>0.93415957460087595</v>
+        <v>0.97842863531828816</v>
       </c>
       <c r="E41"/>
       <c r="O41" s="24">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="P41" s="15">
         <f t="shared" si="0"/>
-        <v>0.93415957460087595</v>
+        <v>0.97842863531828816</v>
       </c>
       <c r="Q41" s="16">
         <f t="shared" si="1"/>
-        <v>3.6075514634148341E-2</v>
+        <v>1.902355381396259E-2</v>
       </c>
       <c r="R41" s="17">
         <f t="shared" si="2"/>
-        <v>1.803775731707417E-2</v>
+        <v>9.5117769069812952E-3</v>
       </c>
       <c r="S41" s="18">
         <f t="shared" si="4"/>
-        <v>0.94924176078785538</v>
+        <v>0.97979149449115144</v>
       </c>
       <c r="T41" s="18">
         <f t="shared" si="3"/>
-        <v>5.0758239212144618E-2</v>
+        <v>2.0208505508848562E-2</v>
       </c>
       <c r="AJ41"/>
       <c r="AK41"/>
@@ -4463,38 +4515,38 @@
       <c r="AP41"/>
       <c r="AQ41"/>
       <c r="AR41"/>
-      <c r="AT41" s="40"/>
+      <c r="AT41" s="39"/>
     </row>
     <row r="42" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C42" s="20">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D42" s="21">
-        <v>0.90105992042362804</v>
+        <v>0.95999137267720414</v>
       </c>
       <c r="E42"/>
       <c r="O42" s="24">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P42" s="15">
         <f t="shared" si="0"/>
-        <v>0.90105992042362804</v>
+        <v>0.95999137267720414</v>
       </c>
       <c r="Q42" s="16">
         <f t="shared" si="1"/>
-        <v>4.4951698721086432E-2</v>
+        <v>2.7277023241003562E-2</v>
       </c>
       <c r="R42" s="17">
         <f t="shared" si="2"/>
-        <v>2.2475849360543216E-2</v>
+        <v>1.3638511620501781E-2</v>
       </c>
       <c r="S42" s="18">
         <f t="shared" si="4"/>
-        <v>0.92814472102375822</v>
+        <v>0.9665193089643247</v>
       </c>
       <c r="T42" s="18">
         <f t="shared" si="3"/>
-        <v>7.1855278976241777E-2</v>
+        <v>3.3480691035675303E-2</v>
       </c>
       <c r="AJ42"/>
       <c r="AK42"/>
@@ -4505,38 +4557,38 @@
       <c r="AP42"/>
       <c r="AQ42"/>
       <c r="AR42"/>
-      <c r="AT42" s="40"/>
+      <c r="AT42" s="39"/>
     </row>
     <row r="43" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C43" s="20">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D43" s="21">
-        <v>0.86145262316426996</v>
+        <v>0.93415957460087595</v>
       </c>
       <c r="E43"/>
       <c r="O43" s="24">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P43" s="15">
         <f t="shared" si="0"/>
-        <v>0.86145262316426996</v>
+        <v>0.93415957460087595</v>
       </c>
       <c r="Q43" s="16">
         <f t="shared" si="1"/>
-        <v>5.3562670757796235E-2</v>
+        <v>3.6075514634148341E-2</v>
       </c>
       <c r="R43" s="17">
         <f t="shared" si="2"/>
-        <v>2.6781335378898118E-2</v>
+        <v>1.803775731707417E-2</v>
       </c>
       <c r="S43" s="18">
         <f t="shared" si="4"/>
-        <v>0.90361766558309942</v>
+        <v>0.94924176078785538</v>
       </c>
       <c r="T43" s="18">
         <f t="shared" si="3"/>
-        <v>9.6382334416900584E-2</v>
+        <v>5.0758239212144618E-2</v>
       </c>
       <c r="AJ43"/>
       <c r="AK43"/>
@@ -4547,38 +4599,38 @@
       <c r="AP43"/>
       <c r="AQ43"/>
       <c r="AR43"/>
-      <c r="AT43" s="40"/>
+      <c r="AT43" s="39"/>
     </row>
     <row r="44" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C44" s="20">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D44" s="21">
-        <v>0.81652488555384994</v>
+        <v>0.90105992042362804</v>
       </c>
       <c r="E44"/>
       <c r="O44" s="24">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P44" s="15">
         <f t="shared" si="0"/>
-        <v>0.81652488555384994</v>
+        <v>0.90105992042362804</v>
       </c>
       <c r="Q44" s="16">
         <f t="shared" si="1"/>
-        <v>6.1685627022741121E-2</v>
+        <v>4.4951698721086432E-2</v>
       </c>
       <c r="R44" s="17">
         <f t="shared" si="2"/>
-        <v>3.0842813511370561E-2</v>
+        <v>2.2475849360543216E-2</v>
       </c>
       <c r="S44" s="18">
         <f t="shared" si="4"/>
-        <v>0.87617296591124472</v>
+        <v>0.92814472102375822</v>
       </c>
       <c r="T44" s="18">
         <f t="shared" si="3"/>
-        <v>0.12382703408875528</v>
+        <v>7.1855278976241777E-2</v>
       </c>
       <c r="AJ44"/>
       <c r="AK44"/>
@@ -4589,38 +4641,38 @@
       <c r="AP44"/>
       <c r="AQ44"/>
       <c r="AR44"/>
-      <c r="AT44" s="40"/>
+      <c r="AT44" s="39"/>
     </row>
     <row r="45" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C45" s="20">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D45" s="21">
-        <v>0.76767906619370696</v>
+        <v>0.86145262316426996</v>
       </c>
       <c r="E45"/>
       <c r="O45" s="24">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="P45" s="15">
         <f t="shared" si="0"/>
-        <v>0.76767906619370696</v>
+        <v>0.86145262316426996</v>
       </c>
       <c r="Q45" s="16">
         <f t="shared" si="1"/>
-        <v>6.9194610516950139E-2</v>
+        <v>5.3562670757796235E-2</v>
       </c>
       <c r="R45" s="17">
         <f t="shared" si="2"/>
-        <v>3.459730525847507E-2</v>
+        <v>2.6781335378898118E-2</v>
       </c>
       <c r="S45" s="18">
         <f t="shared" si="4"/>
-        <v>0.84637812486615904</v>
+        <v>0.90361766558309942</v>
       </c>
       <c r="T45" s="18">
         <f t="shared" si="3"/>
-        <v>0.15362187513384096</v>
+        <v>9.6382334416900584E-2</v>
       </c>
       <c r="AJ45"/>
       <c r="AK45"/>
@@ -4631,38 +4683,38 @@
       <c r="AP45"/>
       <c r="AQ45"/>
       <c r="AR45"/>
-      <c r="AT45" s="40"/>
+      <c r="AT45" s="39"/>
     </row>
     <row r="46" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C46" s="20">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D46" s="21">
-        <v>0.71635593025195532</v>
+        <v>0.81652488555384994</v>
       </c>
       <c r="E46"/>
       <c r="O46" s="24">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="P46" s="15">
         <f t="shared" si="0"/>
-        <v>0.71635593025195532</v>
+        <v>0.81652488555384994</v>
       </c>
       <c r="Q46" s="16">
         <f t="shared" si="1"/>
-        <v>7.6033935478792808E-2</v>
+        <v>6.1685627022741121E-2</v>
       </c>
       <c r="R46" s="17">
         <f t="shared" si="2"/>
-        <v>3.8016967739396404E-2</v>
+        <v>3.0842813511370561E-2</v>
       </c>
       <c r="S46" s="18">
         <f t="shared" si="4"/>
-        <v>0.8148053481737787</v>
+        <v>0.87617296591124472</v>
       </c>
       <c r="T46" s="18">
         <f t="shared" si="3"/>
-        <v>0.1851946518262213</v>
+        <v>0.12382703408875528</v>
       </c>
       <c r="AJ46"/>
       <c r="AK46"/>
@@ -4673,38 +4725,38 @@
       <c r="AP46"/>
       <c r="AQ46"/>
       <c r="AR46"/>
-      <c r="AT46" s="40"/>
+      <c r="AT46" s="39"/>
     </row>
     <row r="47" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C47" s="20">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D47" s="21">
-        <v>0.6639077554125925</v>
+        <v>0.76767906619370696</v>
       </c>
       <c r="E47"/>
       <c r="O47" s="24">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="P47" s="15">
         <f t="shared" si="0"/>
-        <v>0.6639077554125925</v>
+        <v>0.76767906619370696</v>
       </c>
       <c r="Q47" s="16">
         <f t="shared" si="1"/>
-        <v>8.2195135179689766E-2</v>
+        <v>6.9194610516950139E-2</v>
       </c>
       <c r="R47" s="17">
         <f t="shared" si="2"/>
-        <v>4.1097567589844883E-2</v>
+        <v>3.459730525847507E-2</v>
       </c>
       <c r="S47" s="18">
         <f t="shared" si="4"/>
-        <v>0.7819976070704564</v>
+        <v>0.84637812486615904</v>
       </c>
       <c r="T47" s="18">
         <f t="shared" si="3"/>
-        <v>0.2180023929295436</v>
+        <v>0.15362187513384096</v>
       </c>
       <c r="AJ47"/>
       <c r="AK47"/>
@@ -4715,38 +4767,38 @@
       <c r="AP47"/>
       <c r="AQ47"/>
       <c r="AR47"/>
-      <c r="AT47" s="40"/>
+      <c r="AT47" s="39"/>
     </row>
     <row r="48" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C48" s="20">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D48" s="21">
-        <v>0.6115202574639198</v>
+        <v>0.71635593025195532</v>
       </c>
       <c r="E48"/>
       <c r="O48" s="24">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="P48" s="15">
         <f t="shared" si="0"/>
-        <v>0.6115202574639198</v>
+        <v>0.71635593025195532</v>
       </c>
       <c r="Q48" s="16">
         <f t="shared" si="1"/>
-        <v>8.769933078081292E-2</v>
+        <v>7.6033935478792808E-2</v>
       </c>
       <c r="R48" s="17">
         <f t="shared" si="2"/>
-        <v>4.384966539040646E-2</v>
+        <v>3.8016967739396404E-2</v>
       </c>
       <c r="S48" s="18">
         <f t="shared" si="4"/>
-        <v>0.74844821403335726</v>
+        <v>0.8148053481737787</v>
       </c>
       <c r="T48" s="18">
         <f t="shared" si="3"/>
-        <v>0.25155178596664274</v>
+        <v>0.1851946518262213</v>
       </c>
       <c r="AJ48"/>
       <c r="AK48"/>
@@ -4757,38 +4809,38 @@
       <c r="AP48"/>
       <c r="AQ48"/>
       <c r="AR48"/>
-      <c r="AT48" s="40"/>
+      <c r="AT48" s="39"/>
     </row>
     <row r="49" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C49" s="20">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D49" s="21">
-        <v>0.5601747290897221</v>
+        <v>0.6639077554125925</v>
       </c>
       <c r="E49"/>
       <c r="O49" s="24">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="P49" s="15">
         <f t="shared" si="0"/>
-        <v>0.5601747290897221</v>
+        <v>0.6639077554125925</v>
       </c>
       <c r="Q49" s="16">
         <f t="shared" si="1"/>
-        <v>9.2584710801622019E-2</v>
+        <v>8.2195135179689766E-2</v>
       </c>
       <c r="R49" s="17">
         <f t="shared" si="2"/>
-        <v>4.629235540081101E-2</v>
+        <v>4.1097567589844883E-2</v>
       </c>
       <c r="S49" s="18">
         <f t="shared" si="4"/>
-        <v>0.71459050599315621</v>
+        <v>0.7819976070704564</v>
       </c>
       <c r="T49" s="18">
         <f t="shared" si="3"/>
-        <v>0.28540949400684379</v>
+        <v>0.2180023929295436</v>
       </c>
       <c r="AJ49"/>
       <c r="AK49"/>
@@ -4799,38 +4851,38 @@
       <c r="AP49"/>
       <c r="AQ49"/>
       <c r="AR49"/>
-      <c r="AT49" s="40"/>
+      <c r="AT49" s="39"/>
     </row>
     <row r="50" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C50" s="20">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D50" s="21">
-        <v>0.51063959125555491</v>
+        <v>0.6115202574639198</v>
       </c>
       <c r="E50"/>
       <c r="O50" s="24">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="P50" s="15">
         <f t="shared" si="0"/>
-        <v>0.51063959125555491</v>
+        <v>0.6115202574639198</v>
       </c>
       <c r="Q50" s="16">
         <f t="shared" si="1"/>
-        <v>9.6898088907587263E-2</v>
+        <v>8.769933078081292E-2</v>
       </c>
       <c r="R50" s="17">
         <f t="shared" si="2"/>
-        <v>4.8449044453793631E-2</v>
+        <v>4.384966539040646E-2</v>
       </c>
       <c r="S50" s="18">
         <f t="shared" si="4"/>
-        <v>0.6807945795084881</v>
+        <v>0.74844821403335726</v>
       </c>
       <c r="T50" s="18">
         <f t="shared" si="3"/>
-        <v>0.3192054204915119</v>
+        <v>0.25155178596664274</v>
       </c>
       <c r="AJ50"/>
       <c r="AK50"/>
@@ -4841,38 +4893,38 @@
       <c r="AP50"/>
       <c r="AQ50"/>
       <c r="AR50"/>
-      <c r="AT50" s="40"/>
+      <c r="AT50" s="39"/>
     </row>
     <row r="51" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C51" s="20">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D51" s="21">
-        <v>0.46348125948813901</v>
+        <v>0.5601747290897221</v>
       </c>
       <c r="E51"/>
       <c r="O51" s="24">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="P51" s="15">
         <f t="shared" si="0"/>
-        <v>0.46348125948813901</v>
+        <v>0.5601747290897221</v>
       </c>
       <c r="Q51" s="16">
         <f t="shared" si="1"/>
-        <v>0.1006894518792652</v>
+        <v>9.2584710801622019E-2</v>
       </c>
       <c r="R51" s="17">
         <f t="shared" si="2"/>
-        <v>5.0344725939632601E-2</v>
+        <v>4.629235540081101E-2</v>
       </c>
       <c r="S51" s="18">
         <f t="shared" si="4"/>
-        <v>0.64736863283905932</v>
+        <v>0.71459050599315621</v>
       </c>
       <c r="T51" s="18">
         <f t="shared" si="3"/>
-        <v>0.35263136716094068</v>
+        <v>0.28540949400684379</v>
       </c>
       <c r="AJ51"/>
       <c r="AK51"/>
@@ -4883,38 +4935,38 @@
       <c r="AP51"/>
       <c r="AQ51"/>
       <c r="AR51"/>
-      <c r="AT51" s="40"/>
+      <c r="AT51" s="39"/>
     </row>
     <row r="52" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C52" s="20">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D52" s="21">
-        <v>0.41908614678391276</v>
+        <v>0.51063959125555491</v>
       </c>
       <c r="E52"/>
       <c r="O52" s="24">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="P52" s="15">
         <f t="shared" si="0"/>
-        <v>0.41908614678391276</v>
+        <v>0.51063959125555491</v>
       </c>
       <c r="Q52" s="16">
         <f t="shared" si="1"/>
-        <v>0.10400859015696973</v>
+        <v>9.6898088907587263E-2</v>
       </c>
       <c r="R52" s="17">
         <f t="shared" si="2"/>
-        <v>5.2004295078484863E-2</v>
+        <v>4.8449044453793631E-2</v>
       </c>
       <c r="S52" s="18">
         <f t="shared" si="4"/>
-        <v>0.61456309104035634</v>
+        <v>0.6807945795084881</v>
       </c>
       <c r="T52" s="18">
         <f t="shared" si="3"/>
-        <v>0.38543690895964366</v>
+        <v>0.3192054204915119</v>
       </c>
       <c r="AJ52"/>
       <c r="AK52"/>
@@ -4925,38 +4977,38 @@
       <c r="AP52"/>
       <c r="AQ52"/>
       <c r="AR52"/>
-      <c r="AT52" s="40"/>
+      <c r="AT52" s="39"/>
     </row>
     <row r="53" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C53" s="20">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D53" s="21">
-        <v>0.37768779286907717</v>
+        <v>0.46348125948813901</v>
       </c>
       <c r="E53"/>
       <c r="O53" s="24">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="P53" s="15">
         <f t="shared" si="0"/>
-        <v>0.37768779286907717</v>
+        <v>0.46348125948813901</v>
       </c>
       <c r="Q53" s="16">
         <f t="shared" si="1"/>
-        <v>0.10690312815263153</v>
+        <v>0.1006894518792652</v>
       </c>
       <c r="R53" s="17">
         <f t="shared" si="2"/>
-        <v>5.3451564076315766E-2</v>
+        <v>5.0344725939632601E-2</v>
       </c>
       <c r="S53" s="18">
         <f t="shared" si="4"/>
-        <v>0.5825762220528844</v>
+        <v>0.64736863283905932</v>
       </c>
       <c r="T53" s="18">
         <f t="shared" si="3"/>
-        <v>0.4174237779471156</v>
+        <v>0.35263136716094068</v>
       </c>
       <c r="AJ53"/>
       <c r="AK53"/>
@@ -4967,38 +5019,38 @@
       <c r="AP53"/>
       <c r="AQ53"/>
       <c r="AR53"/>
-      <c r="AT53" s="40"/>
+      <c r="AT53" s="39"/>
     </row>
     <row r="54" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C54" s="20">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D54" s="21">
-        <v>0.3393950545014115</v>
+        <v>0.41908614678391276</v>
       </c>
       <c r="E54"/>
       <c r="O54" s="24">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="P54" s="15">
         <f t="shared" si="0"/>
-        <v>0.3393950545014115</v>
+        <v>0.41908614678391276</v>
       </c>
       <c r="Q54" s="16">
         <f t="shared" si="1"/>
-        <v>0.10941746904383318</v>
+        <v>0.10400859015696973</v>
       </c>
       <c r="R54" s="17">
         <f t="shared" si="2"/>
-        <v>5.4708734521916588E-2</v>
+        <v>5.2004295078484863E-2</v>
       </c>
       <c r="S54" s="18">
         <f t="shared" si="4"/>
-        <v>0.55156036882472337</v>
+        <v>0.61456309104035634</v>
       </c>
       <c r="T54" s="18">
         <f t="shared" si="3"/>
-        <v>0.44843963117527663</v>
+        <v>0.38543690895964366</v>
       </c>
       <c r="AJ54"/>
       <c r="AK54"/>
@@ -5009,38 +5061,38 @@
       <c r="AP54"/>
       <c r="AQ54"/>
       <c r="AR54"/>
-      <c r="AT54" s="40"/>
+      <c r="AT54" s="39"/>
     </row>
     <row r="55" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C55" s="20">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D55" s="21">
-        <v>0.30421884045806469</v>
+        <v>0.37768779286907717</v>
       </c>
       <c r="E55"/>
       <c r="O55" s="24">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="P55" s="15">
         <f t="shared" si="0"/>
-        <v>0.30421884045806469</v>
+        <v>0.37768779286907717</v>
       </c>
       <c r="Q55" s="16">
         <f t="shared" si="1"/>
-        <v>0.11159232117592577</v>
+        <v>0.10690312815263153</v>
       </c>
       <c r="R55" s="17">
         <f t="shared" si="2"/>
-        <v>5.5796160587962884E-2</v>
+        <v>5.3451564076315766E-2</v>
       </c>
       <c r="S55" s="18">
         <f t="shared" si="4"/>
-        <v>0.52162823208582532</v>
+        <v>0.5825762220528844</v>
       </c>
       <c r="T55" s="18">
         <f t="shared" si="3"/>
-        <v>0.47837176791417468</v>
+        <v>0.4174237779471156</v>
       </c>
       <c r="AJ55"/>
       <c r="AK55"/>
@@ -5051,38 +5103,38 @@
       <c r="AP55"/>
       <c r="AQ55"/>
       <c r="AR55"/>
-      <c r="AT55" s="40"/>
+      <c r="AT55" s="39"/>
     </row>
     <row r="56" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C56" s="20">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D56" s="21">
-        <v>0.27209601250898352</v>
+        <v>0.3393950545014115</v>
       </c>
       <c r="E56"/>
       <c r="O56" s="24">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="P56" s="15">
         <f t="shared" si="0"/>
-        <v>0.27209601250898352</v>
+        <v>0.3393950545014115</v>
       </c>
       <c r="Q56" s="16">
         <f t="shared" si="1"/>
-        <v>0.1134645832848865</v>
+        <v>0.10941746904383318</v>
       </c>
       <c r="R56" s="17">
         <f t="shared" si="2"/>
-        <v>5.6732291642443249E-2</v>
+        <v>5.4708734521916588E-2</v>
       </c>
       <c r="S56" s="18">
         <f t="shared" si="4"/>
-        <v>0.49285885921865324</v>
+        <v>0.55156036882472337</v>
       </c>
       <c r="T56" s="18">
         <f t="shared" si="3"/>
-        <v>0.50714114078134676</v>
+        <v>0.44843963117527663</v>
       </c>
       <c r="AJ56"/>
       <c r="AK56"/>
@@ -5093,38 +5145,38 @@
       <c r="AP56"/>
       <c r="AQ56"/>
       <c r="AR56"/>
-      <c r="AT56" s="40"/>
+      <c r="AT56" s="39"/>
     </row>
     <row r="57" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C57" s="20">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D57" s="21">
-        <v>0.24290985511031216</v>
+        <v>0.30421884045806469</v>
       </c>
       <c r="E57"/>
       <c r="O57" s="24">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="P57" s="15">
         <f t="shared" si="0"/>
-        <v>0.24290985511031216</v>
+        <v>0.30421884045806469</v>
       </c>
       <c r="Q57" s="16">
         <f t="shared" si="1"/>
-        <v>0.11506744226367967</v>
+        <v>0.11159232117592577</v>
       </c>
       <c r="R57" s="17">
         <f t="shared" si="2"/>
-        <v>5.7533721131839834E-2</v>
+        <v>5.5796160587962884E-2</v>
       </c>
       <c r="S57" s="18">
         <f t="shared" si="4"/>
-        <v>0.46530314704588888</v>
+        <v>0.52162823208582532</v>
       </c>
       <c r="T57" s="18">
         <f t="shared" si="3"/>
-        <v>0.53469685295411118</v>
+        <v>0.47837176791417468</v>
       </c>
       <c r="AJ57"/>
       <c r="AK57"/>
@@ -5135,38 +5187,38 @@
       <c r="AP57"/>
       <c r="AQ57"/>
       <c r="AR57"/>
-      <c r="AT57" s="40"/>
+      <c r="AT57" s="39"/>
     </row>
     <row r="58" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C58" s="20">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D58" s="21">
-        <v>0.21650701865080801</v>
+        <v>0.27209601250898352</v>
       </c>
       <c r="E58"/>
       <c r="O58" s="24">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="P58" s="15">
         <f t="shared" si="0"/>
-        <v>0.21650701865080801</v>
+        <v>0.27209601250898352</v>
       </c>
       <c r="Q58" s="16">
         <f t="shared" si="1"/>
-        <v>0.11643058907955031</v>
+        <v>0.1134645832848865</v>
       </c>
       <c r="R58" s="17">
         <f t="shared" si="2"/>
-        <v>5.8215294539775156E-2</v>
+        <v>5.6732291642443249E-2</v>
       </c>
       <c r="S58" s="18">
         <f t="shared" si="4"/>
-        <v>0.43898876819253896</v>
+        <v>0.49285885921865324</v>
       </c>
       <c r="T58" s="18">
         <f t="shared" si="3"/>
-        <v>0.56101123180746104</v>
+        <v>0.50714114078134676</v>
       </c>
       <c r="AJ58"/>
       <c r="AK58"/>
@@ -5177,38 +5229,38 @@
       <c r="AP58"/>
       <c r="AQ58"/>
       <c r="AR58"/>
-      <c r="AT58" s="40"/>
+      <c r="AT58" s="39"/>
     </row>
     <row r="59" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C59" s="20">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D59" s="21">
-        <v>0.19271113859920264</v>
+        <v>0.24290985511031216</v>
       </c>
       <c r="E59"/>
       <c r="O59" s="24">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="P59" s="15">
         <f t="shared" si="0"/>
-        <v>0.19271113859920264</v>
+        <v>0.24290985511031216</v>
       </c>
       <c r="Q59" s="16">
         <f t="shared" si="1"/>
-        <v>0.11758049304174645</v>
+        <v>0.11506744226367967</v>
       </c>
       <c r="R59" s="17">
         <f t="shared" si="2"/>
-        <v>5.8790246520873224E-2</v>
+        <v>5.7533721131839834E-2</v>
       </c>
       <c r="S59" s="18">
         <f t="shared" si="4"/>
-        <v>0.41392449635726764</v>
+        <v>0.46530314704588888</v>
       </c>
       <c r="T59" s="18">
         <f t="shared" si="3"/>
-        <v>0.58607550364273231</v>
+        <v>0.53469685295411118</v>
       </c>
       <c r="AJ59"/>
       <c r="AK59"/>
@@ -5219,38 +5271,38 @@
       <c r="AP59"/>
       <c r="AQ59"/>
       <c r="AR59"/>
-      <c r="AT59" s="40"/>
+      <c r="AT59" s="39"/>
     </row>
     <row r="60" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C60" s="20">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D60" s="21">
-        <v>0.17133348868461762</v>
+        <v>0.21650701865080801</v>
       </c>
       <c r="E60"/>
       <c r="O60" s="24">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="P60" s="15">
         <f t="shared" si="0"/>
-        <v>0.17133348868461762</v>
+        <v>0.21650701865080801</v>
       </c>
       <c r="Q60" s="16">
         <f t="shared" si="1"/>
-        <v>0.11854069738435768</v>
+        <v>0.11643058907955031</v>
       </c>
       <c r="R60" s="17">
         <f t="shared" si="2"/>
-        <v>5.9270348692178842E-2</v>
+        <v>5.8215294539775156E-2</v>
       </c>
       <c r="S60" s="18">
         <f t="shared" si="4"/>
-        <v>0.39010394628692258</v>
+        <v>0.43898876819253896</v>
       </c>
       <c r="T60" s="18">
         <f t="shared" si="3"/>
-        <v>0.60989605371307742</v>
+        <v>0.56101123180746104</v>
       </c>
       <c r="AJ60"/>
       <c r="AK60"/>
@@ -5261,38 +5313,38 @@
       <c r="AP60"/>
       <c r="AQ60"/>
       <c r="AR60"/>
-      <c r="AT60" s="40"/>
+      <c r="AT60" s="39"/>
     </row>
     <row r="61" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C61" s="20">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D61" s="21">
-        <v>0.15218108890863014</v>
+        <v>0.19271113859920264</v>
       </c>
       <c r="E61"/>
       <c r="O61" s="24">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="P61" s="15">
         <f t="shared" si="0"/>
-        <v>0.15218108890863014</v>
+        <v>0.19271113859920264</v>
       </c>
       <c r="Q61" s="16">
         <f t="shared" si="1"/>
-        <v>0.11933211394118085</v>
+        <v>0.11758049304174645</v>
       </c>
       <c r="R61" s="17">
         <f t="shared" si="2"/>
-        <v>5.9666056970590423E-2</v>
+        <v>5.8790246520873224E-2</v>
       </c>
       <c r="S61" s="18">
         <f t="shared" si="4"/>
-        <v>0.36750876752580985</v>
+        <v>0.41392449635726764</v>
       </c>
       <c r="T61" s="18">
         <f t="shared" si="3"/>
-        <v>0.63249123247419015</v>
+        <v>0.58607550364273231</v>
       </c>
       <c r="AJ61"/>
       <c r="AK61"/>
@@ -5303,38 +5355,38 @@
       <c r="AP61"/>
       <c r="AQ61"/>
       <c r="AR61"/>
-      <c r="AT61" s="40"/>
+      <c r="AT61" s="39"/>
     </row>
     <row r="62" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C62" s="20">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D62" s="21">
-        <v>0.13506269420833972</v>
+        <v>0.17133348868461762</v>
       </c>
       <c r="E62"/>
       <c r="O62" s="24">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="P62" s="15">
         <f t="shared" si="0"/>
-        <v>0.13506269420833972</v>
+        <v>0.17133348868461762</v>
       </c>
       <c r="Q62" s="16">
         <f t="shared" si="1"/>
-        <v>0.11997330421583355</v>
+        <v>0.11854069738435768</v>
       </c>
       <c r="R62" s="17">
         <f t="shared" si="2"/>
-        <v>5.9986652107916774E-2</v>
+        <v>5.9270348692178842E-2</v>
       </c>
       <c r="S62" s="18">
         <f t="shared" si="4"/>
-        <v>0.34611134286308715</v>
+        <v>0.39010394628692258</v>
       </c>
       <c r="T62" s="18">
         <f t="shared" si="3"/>
-        <v>0.65388865713691291</v>
+        <v>0.60989605371307742</v>
       </c>
       <c r="AJ62"/>
       <c r="AK62"/>
@@ -5345,38 +5397,38 @@
       <c r="AP62"/>
       <c r="AQ62"/>
       <c r="AR62"/>
-      <c r="AT62" s="40"/>
+      <c r="AT62" s="39"/>
     </row>
     <row r="63" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C63" s="20">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D63" s="21">
-        <v>0.11979306165848946</v>
+        <v>0.15218108890863014</v>
       </c>
       <c r="E63"/>
       <c r="O63" s="24">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="P63" s="15">
         <f t="shared" si="0"/>
-        <v>0.11979306165848946</v>
+        <v>0.15218108890863014</v>
       </c>
       <c r="Q63" s="16">
         <f t="shared" si="1"/>
-        <v>0.12048074019441422</v>
+        <v>0.11933211394118085</v>
       </c>
       <c r="R63" s="17">
         <f t="shared" si="2"/>
-        <v>6.0240370097207112E-2</v>
+        <v>5.9666056970590423E-2</v>
       </c>
       <c r="S63" s="18">
         <f t="shared" si="4"/>
-        <v>0.3258770468672591</v>
+        <v>0.36750876752580985</v>
       </c>
       <c r="T63" s="18">
         <f t="shared" si="3"/>
-        <v>0.67412295313274084</v>
+        <v>0.63249123247419015</v>
       </c>
       <c r="AJ63"/>
       <c r="AK63"/>
@@ -5387,38 +5439,38 @@
       <c r="AP63"/>
       <c r="AQ63"/>
       <c r="AR63"/>
-      <c r="AT63" s="40"/>
+      <c r="AT63" s="39"/>
     </row>
     <row r="64" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C64" s="20">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D64" s="21">
-        <v>0.10619584967492579</v>
+        <v>0.13506269420833972</v>
       </c>
       <c r="E64"/>
       <c r="O64" s="24">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="P64" s="15">
         <f t="shared" si="0"/>
-        <v>0.10619584967492579</v>
+        <v>0.13506269420833972</v>
       </c>
       <c r="Q64" s="16">
         <f t="shared" si="1"/>
-        <v>0.12086904201425032</v>
+        <v>0.11997330421583355</v>
       </c>
       <c r="R64" s="17">
         <f t="shared" si="2"/>
-        <v>6.043452100712516E-2</v>
+        <v>5.9986652107916774E-2</v>
       </c>
       <c r="S64" s="18">
         <f t="shared" si="4"/>
-        <v>0.30676611976122475</v>
+        <v>0.34611134286308715</v>
       </c>
       <c r="T64" s="18">
         <f t="shared" si="3"/>
-        <v>0.69323388023877519</v>
+        <v>0.65388865713691291</v>
       </c>
       <c r="AJ64"/>
       <c r="AK64"/>
@@ -5429,38 +5481,38 @@
       <c r="AP64"/>
       <c r="AQ64"/>
       <c r="AR64"/>
-      <c r="AT64" s="40"/>
+      <c r="AT64" s="39"/>
     </row>
     <row r="65" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C65" s="20">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D65" s="21">
-        <v>9.4105452233358089E-2</v>
+        <v>0.11979306165848946</v>
       </c>
       <c r="E65"/>
       <c r="O65" s="24">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="P65" s="15">
         <f t="shared" si="0"/>
-        <v>9.4105452233358089E-2</v>
+        <v>0.11979306165848946</v>
       </c>
       <c r="Q65" s="16">
         <f t="shared" si="1"/>
-        <v>0.1211511918902398</v>
+        <v>0.12048074019441422</v>
       </c>
       <c r="R65" s="17">
         <f t="shared" si="2"/>
-        <v>6.0575595945119902E-2</v>
+        <v>6.0240370097207112E-2</v>
       </c>
       <c r="S65" s="18">
         <f t="shared" si="4"/>
-        <v>0.28873520904113287</v>
+        <v>0.3258770468672591</v>
       </c>
       <c r="T65" s="18">
         <f t="shared" si="3"/>
-        <v>0.71126479095886719</v>
+        <v>0.67412295313274084</v>
       </c>
       <c r="AJ65"/>
       <c r="AK65"/>
@@ -5471,38 +5523,38 @@
       <c r="AP65"/>
       <c r="AQ65"/>
       <c r="AR65"/>
-      <c r="AT65" s="40"/>
+      <c r="AT65" s="39"/>
     </row>
     <row r="66" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C66" s="20">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D66" s="21">
-        <v>8.336802094002671E-2</v>
+        <v>0.10619584967492579</v>
       </c>
       <c r="E66"/>
       <c r="O66" s="24">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="P66" s="15">
         <f t="shared" si="0"/>
-        <v>8.336802094002671E-2</v>
+        <v>0.10619584967492579</v>
       </c>
       <c r="Q66" s="16">
         <f t="shared" si="1"/>
-        <v>0.12133872503625612</v>
+        <v>0.12086904201425032</v>
       </c>
       <c r="R66" s="17">
         <f t="shared" si="2"/>
-        <v>6.0669362518128059E-2</v>
+        <v>6.043452100712516E-2</v>
       </c>
       <c r="S66" s="18">
         <f t="shared" si="4"/>
-        <v>0.27173862693106593</v>
+        <v>0.30676611976122475</v>
       </c>
       <c r="T66" s="18">
         <f t="shared" si="3"/>
-        <v>0.72826137306893401</v>
+        <v>0.69323388023877519</v>
       </c>
       <c r="AJ66"/>
       <c r="AK66"/>
@@ -5513,38 +5565,38 @@
       <c r="AP66"/>
       <c r="AQ66"/>
       <c r="AR66"/>
-      <c r="AT66" s="40"/>
+      <c r="AT66" s="39"/>
     </row>
     <row r="67" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C67" s="20">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D67" s="21">
-        <v>7.3841881366381035E-2</v>
+        <v>9.4105452233358089E-2</v>
       </c>
       <c r="E67"/>
       <c r="O67" s="24">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="P67" s="15">
         <f t="shared" si="0"/>
-        <v>7.3841881366381035E-2</v>
+        <v>9.4105452233358089E-2</v>
       </c>
       <c r="Q67" s="16">
         <f t="shared" si="1"/>
-        <v>0.12144189904880337</v>
+        <v>0.1211511918902398</v>
       </c>
       <c r="R67" s="17">
         <f t="shared" si="2"/>
-        <v>6.0720949524401685E-2</v>
+        <v>6.0575595945119902E-2</v>
       </c>
       <c r="S67" s="18">
         <f t="shared" si="4"/>
-        <v>0.25572936680721148</v>
+        <v>0.28873520904113287</v>
       </c>
       <c r="T67" s="18">
         <f t="shared" si="3"/>
-        <v>0.74427063319278852</v>
+        <v>0.71126479095886719</v>
       </c>
       <c r="AJ67"/>
       <c r="AK67"/>
@@ -5555,38 +5607,38 @@
       <c r="AP67"/>
       <c r="AQ67"/>
       <c r="AR67"/>
-      <c r="AT67" s="40"/>
+      <c r="AT67" s="39"/>
     </row>
     <row r="68" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C68" s="20">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D68" s="21">
-        <v>6.5397509047617319E-2</v>
+        <v>8.336802094002671E-2</v>
       </c>
       <c r="E68"/>
       <c r="O68" s="24">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="P68" s="15">
         <f t="shared" si="0"/>
-        <v>6.5397509047617319E-2</v>
+        <v>8.336802094002671E-2</v>
       </c>
       <c r="Q68" s="16">
         <f t="shared" si="1"/>
-        <v>0.12146984356956154</v>
+        <v>0.12133872503625612</v>
       </c>
       <c r="R68" s="17">
         <f t="shared" si="2"/>
-        <v>6.0734921784780772E-2</v>
+        <v>6.0669362518128059E-2</v>
       </c>
       <c r="S68" s="18">
         <f t="shared" si="4"/>
-        <v>0.24065991663219075</v>
+        <v>0.27173862693106593</v>
       </c>
       <c r="T68" s="18">
         <f t="shared" si="3"/>
-        <v>0.75934008336780923</v>
+        <v>0.72826137306893401</v>
       </c>
       <c r="AJ68"/>
       <c r="AK68"/>
@@ -5597,38 +5649,38 @@
       <c r="AP68"/>
       <c r="AQ68"/>
       <c r="AR68"/>
-      <c r="AT68" s="40"/>
+      <c r="AT68" s="39"/>
     </row>
     <row r="69" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C69" s="20">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D69" s="21">
-        <v>5.7917195473413008E-2</v>
+        <v>7.3841881366381035E-2</v>
       </c>
       <c r="E69"/>
       <c r="O69" s="24">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="P69" s="15">
         <f t="shared" si="0"/>
-        <v>5.7917195473413008E-2</v>
+        <v>7.3841881366381035E-2</v>
       </c>
       <c r="Q69" s="16">
         <f t="shared" si="1"/>
-        <v>0.1214306921588577</v>
+        <v>0.12144189904880337</v>
       </c>
       <c r="R69" s="17">
         <f t="shared" si="2"/>
-        <v>6.0715346079428849E-2</v>
+        <v>6.0720949524401685E-2</v>
       </c>
       <c r="S69" s="18">
         <f t="shared" si="4"/>
-        <v>0.22648290252142592</v>
+        <v>0.25572936680721148</v>
       </c>
       <c r="T69" s="18">
         <f t="shared" si="3"/>
-        <v>0.77351709747857411</v>
+        <v>0.74427063319278852</v>
       </c>
       <c r="AJ69"/>
       <c r="AK69"/>
@@ -5639,38 +5691,38 @@
       <c r="AP69"/>
       <c r="AQ69"/>
       <c r="AR69"/>
-      <c r="AT69" s="40"/>
+      <c r="AT69" s="39"/>
     </row>
     <row r="70" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C70" s="20">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D70" s="21">
-        <v>5.1294505134529711E-2</v>
+        <v>6.5397509047617319E-2</v>
       </c>
       <c r="E70"/>
       <c r="O70" s="24">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="P70" s="15">
         <f t="shared" si="0"/>
-        <v>5.1294505134529711E-2</v>
+        <v>6.5397509047617319E-2</v>
       </c>
       <c r="Q70" s="16">
         <f t="shared" si="1"/>
-        <v>0.12133169828870057</v>
+        <v>0.12146984356956154</v>
       </c>
       <c r="R70" s="17">
         <f t="shared" si="2"/>
-        <v>6.0665849144350283E-2</v>
+        <v>6.0734921784780772E-2</v>
       </c>
       <c r="S70" s="18">
         <f t="shared" si="4"/>
-        <v>0.21315159099200889</v>
+        <v>0.24065991663219075</v>
       </c>
       <c r="T70" s="18">
         <f t="shared" si="3"/>
-        <v>0.78684840900799113</v>
+        <v>0.75934008336780923</v>
       </c>
       <c r="AJ70"/>
       <c r="AK70"/>
@@ -5681,38 +5733,38 @@
       <c r="AP70"/>
       <c r="AQ70"/>
       <c r="AR70"/>
-      <c r="AT70" s="40"/>
+      <c r="AT70" s="39"/>
     </row>
     <row r="71" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C71" s="20">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D71" s="21">
-        <v>4.543360074242464E-2</v>
+        <v>5.7917195473413008E-2</v>
       </c>
       <c r="E71"/>
       <c r="O71" s="24">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="P71" s="15">
         <f t="shared" si="0"/>
-        <v>4.543360074242464E-2</v>
+        <v>5.7917195473413008E-2</v>
       </c>
       <c r="Q71" s="16">
         <f t="shared" si="1"/>
-        <v>0.12117933726232513</v>
+        <v>0.1214306921588577</v>
       </c>
       <c r="R71" s="17">
         <f t="shared" si="2"/>
-        <v>6.0589668631162566E-2</v>
+        <v>6.0715346079428849E-2</v>
       </c>
       <c r="S71" s="18">
         <f t="shared" si="4"/>
-        <v>0.20062027430519319</v>
+        <v>0.22648290252142592</v>
       </c>
       <c r="T71" s="18">
         <f t="shared" si="3"/>
-        <v>0.79937972569480675</v>
+        <v>0.77351709747857411</v>
       </c>
       <c r="AJ71"/>
       <c r="AK71"/>
@@ -5723,38 +5775,38 @@
       <c r="AP71"/>
       <c r="AQ71"/>
       <c r="AR71"/>
-      <c r="AT71" s="40"/>
+      <c r="AT71" s="39"/>
     </row>
     <row r="72" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C72" s="20">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D72" s="21">
-        <v>4.0248494462290951E-2</v>
+        <v>5.1294505134529711E-2</v>
       </c>
       <c r="E72"/>
       <c r="O72" s="24">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="P72" s="15">
         <f t="shared" si="0"/>
-        <v>4.0248494462290951E-2</v>
+        <v>5.1294505134529711E-2</v>
       </c>
       <c r="Q72" s="16">
         <f t="shared" si="1"/>
-        <v>0.12097939572523431</v>
+        <v>0.12133169828870057</v>
       </c>
       <c r="R72" s="17">
         <f t="shared" si="2"/>
-        <v>6.0489697862617153E-2</v>
+        <v>6.0665849144350283E-2</v>
       </c>
       <c r="S72" s="18">
         <f t="shared" si="4"/>
-        <v>0.18884455963481769</v>
+        <v>0.21315159099200889</v>
       </c>
       <c r="T72" s="18">
         <f t="shared" si="3"/>
-        <v>0.81115544036518228</v>
+        <v>0.78684840900799113</v>
       </c>
       <c r="AJ72"/>
       <c r="AK72"/>
@@ -5765,38 +5817,38 @@
       <c r="AP72"/>
       <c r="AQ72"/>
       <c r="AR72"/>
-      <c r="AT72" s="40"/>
+      <c r="AT72" s="39"/>
     </row>
     <row r="73" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C73" s="20">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D73" s="21">
-        <v>3.5662267703668205E-2</v>
+        <v>4.543360074242464E-2</v>
       </c>
       <c r="E73"/>
       <c r="O73" s="24">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="P73" s="15">
         <f t="shared" si="0"/>
-        <v>3.5662267703668205E-2</v>
+        <v>4.543360074242464E-2</v>
       </c>
       <c r="Q73" s="16">
         <f t="shared" si="1"/>
-        <v>0.12073705027477381</v>
+        <v>0.12117933726232513</v>
       </c>
       <c r="R73" s="17">
         <f t="shared" si="2"/>
-        <v>6.0368525137386907E-2</v>
+        <v>6.0589668631162566E-2</v>
       </c>
       <c r="S73" s="18">
         <f t="shared" si="4"/>
-        <v>0.17778157956956087</v>
+        <v>0.20062027430519319</v>
       </c>
       <c r="T73" s="18">
         <f t="shared" si="3"/>
-        <v>0.82221842043043913</v>
+        <v>0.79937972569480675</v>
       </c>
       <c r="AJ73"/>
       <c r="AK73"/>
@@ -5807,38 +5859,38 @@
       <c r="AP73"/>
       <c r="AQ73"/>
       <c r="AR73"/>
-      <c r="AT73" s="40"/>
+      <c r="AT73" s="39"/>
     </row>
     <row r="74" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C74" s="20">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D74" s="21">
-        <v>3.1606290034248086E-2</v>
+        <v>4.0248494462290951E-2</v>
       </c>
       <c r="E74"/>
       <c r="O74" s="24">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="P74" s="15">
         <f t="shared" si="0"/>
-        <v>3.1606290034248086E-2</v>
+        <v>4.0248494462290951E-2</v>
       </c>
       <c r="Q74" s="16">
         <f t="shared" si="1"/>
-        <v>0.12045693651537326</v>
+        <v>0.12097939572523431</v>
       </c>
       <c r="R74" s="17">
         <f t="shared" si="2"/>
-        <v>6.0228468257686629E-2</v>
+        <v>6.0489697862617153E-2</v>
       </c>
       <c r="S74" s="18">
         <f t="shared" si="4"/>
-        <v>0.16739013866083813</v>
+        <v>0.18884455963481769</v>
       </c>
       <c r="T74" s="18">
         <f t="shared" si="3"/>
-        <v>0.83260986133916193</v>
+        <v>0.81115544036518228</v>
       </c>
       <c r="AJ74"/>
       <c r="AK74"/>
@@ -5849,38 +5901,38 @@
       <c r="AP74"/>
       <c r="AQ74"/>
       <c r="AR74"/>
-      <c r="AT74" s="40"/>
+      <c r="AT74" s="39"/>
     </row>
     <row r="75" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C75" s="20">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D75" s="21">
-        <v>2.8019458520894602E-2</v>
+        <v>3.5662267703668205E-2</v>
       </c>
       <c r="E75"/>
       <c r="O75" s="24">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="P75" s="15">
         <f t="shared" si="0"/>
-        <v>2.8019458520894602E-2</v>
+        <v>3.5662267703668205E-2</v>
       </c>
       <c r="Q75" s="16">
         <f t="shared" si="1"/>
-        <v>0.1201432097531865</v>
+        <v>0.12073705027477381</v>
       </c>
       <c r="R75" s="17">
         <f t="shared" si="2"/>
-        <v>6.007160487659325E-2</v>
+        <v>6.0368525137386907E-2</v>
       </c>
       <c r="S75" s="18">
         <f t="shared" si="4"/>
-        <v>0.15763080832383303</v>
+        <v>0.17778157956956087</v>
       </c>
       <c r="T75" s="18">
         <f t="shared" si="3"/>
-        <v>0.84236919167616697</v>
+        <v>0.82221842043043913</v>
       </c>
       <c r="AJ75"/>
       <c r="AK75"/>
@@ -5891,38 +5943,38 @@
       <c r="AP75"/>
       <c r="AQ75"/>
       <c r="AR75"/>
-      <c r="AT75" s="40"/>
+      <c r="AT75" s="39"/>
     </row>
     <row r="76" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C76" s="20">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D76" s="21">
-        <v>2.4847471732824977E-2</v>
+        <v>3.1606290034248086E-2</v>
       </c>
       <c r="E76"/>
       <c r="O76" s="24">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="P76" s="15">
         <f t="shared" si="0"/>
-        <v>2.4847471732824977E-2</v>
+        <v>3.1606290034248086E-2</v>
       </c>
       <c r="Q76" s="16">
         <f t="shared" si="1"/>
-        <v>0.11979959838131723</v>
+        <v>0.12045693651537326</v>
       </c>
       <c r="R76" s="17">
         <f t="shared" si="2"/>
-        <v>5.9899799190658617E-2</v>
+        <v>6.0228468257686629E-2</v>
       </c>
       <c r="S76" s="18">
         <f t="shared" si="4"/>
-        <v>0.14846598034570369</v>
+        <v>0.16739013866083813</v>
       </c>
       <c r="T76" s="18">
         <f t="shared" si="3"/>
-        <v>0.85153401965429631</v>
+        <v>0.83260986133916193</v>
       </c>
       <c r="AJ76"/>
       <c r="AK76"/>
@@ -5933,38 +5985,38 @@
       <c r="AP76"/>
       <c r="AQ76"/>
       <c r="AR76"/>
-      <c r="AT76" s="40"/>
+      <c r="AT76" s="39"/>
     </row>
     <row r="77" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C77" s="20">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D77" s="21">
-        <v>2.2042147320010863E-2</v>
+        <v>2.8019458520894602E-2</v>
       </c>
       <c r="E77"/>
       <c r="O77" s="24">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="P77" s="15">
         <f t="shared" si="0"/>
-        <v>2.2042147320010863E-2</v>
-      </c>
-      <c r="Q77" s="16" t="str">
+        <v>2.8019458520894602E-2</v>
+      </c>
+      <c r="Q77" s="16">
         <f t="shared" si="1"/>
-        <v>n/a</v>
-      </c>
-      <c r="R77" s="17" t="str">
+        <v>0.1201432097531865</v>
+      </c>
+      <c r="R77" s="17">
         <f t="shared" si="2"/>
-        <v>n/a</v>
-      </c>
-      <c r="S77" s="18" t="str">
+        <v>6.007160487659325E-2</v>
+      </c>
+      <c r="S77" s="18">
         <f t="shared" si="4"/>
-        <v>n/a</v>
-      </c>
-      <c r="T77" s="18" t="str">
+        <v>0.15763080832383303</v>
+      </c>
+      <c r="T77" s="18">
         <f t="shared" si="3"/>
-        <v>n/a</v>
+        <v>0.84236919167616697</v>
       </c>
       <c r="AJ77"/>
       <c r="AK77"/>
@@ -5975,9 +6027,39 @@
       <c r="AP77"/>
       <c r="AQ77"/>
       <c r="AR77"/>
-      <c r="AT77" s="40"/>
+      <c r="AT77" s="39"/>
     </row>
     <row r="78" spans="3:46" x14ac:dyDescent="0.2">
+      <c r="C78" s="20">
+        <v>49</v>
+      </c>
+      <c r="D78" s="21">
+        <v>2.4847471732824977E-2</v>
+      </c>
+      <c r="E78"/>
+      <c r="O78" s="24">
+        <v>49</v>
+      </c>
+      <c r="P78" s="15">
+        <f t="shared" si="0"/>
+        <v>2.4847471732824977E-2</v>
+      </c>
+      <c r="Q78" s="16">
+        <f t="shared" si="1"/>
+        <v>0.11979959838131723</v>
+      </c>
+      <c r="R78" s="17">
+        <f t="shared" si="2"/>
+        <v>5.9899799190658617E-2</v>
+      </c>
+      <c r="S78" s="18">
+        <f t="shared" si="4"/>
+        <v>0.14846598034570369</v>
+      </c>
+      <c r="T78" s="18">
+        <f t="shared" si="3"/>
+        <v>0.85153401965429631</v>
+      </c>
       <c r="AJ78"/>
       <c r="AK78"/>
       <c r="AL78"/>
@@ -5987,11 +6069,39 @@
       <c r="AP78"/>
       <c r="AQ78"/>
       <c r="AR78"/>
-      <c r="AT78" s="40"/>
+      <c r="AT78" s="39"/>
     </row>
     <row r="79" spans="3:46" x14ac:dyDescent="0.2">
-      <c r="AH79"/>
-      <c r="AI79"/>
+      <c r="C79" s="20">
+        <v>50</v>
+      </c>
+      <c r="D79" s="21">
+        <v>2.2042147320010863E-2</v>
+      </c>
+      <c r="E79"/>
+      <c r="O79" s="24">
+        <v>50</v>
+      </c>
+      <c r="P79" s="15">
+        <f t="shared" si="0"/>
+        <v>2.2042147320010863E-2</v>
+      </c>
+      <c r="Q79" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v>n/a</v>
+      </c>
+      <c r="R79" s="17" t="str">
+        <f t="shared" si="2"/>
+        <v>n/a</v>
+      </c>
+      <c r="S79" s="18" t="str">
+        <f t="shared" si="4"/>
+        <v>n/a</v>
+      </c>
+      <c r="T79" s="18" t="str">
+        <f t="shared" si="3"/>
+        <v>n/a</v>
+      </c>
       <c r="AJ79"/>
       <c r="AK79"/>
       <c r="AL79"/>
@@ -6001,23 +6111,9 @@
       <c r="AP79"/>
       <c r="AQ79"/>
       <c r="AR79"/>
-      <c r="AT79" s="40"/>
+      <c r="AT79" s="39"/>
     </row>
     <row r="80" spans="3:46" x14ac:dyDescent="0.2">
-      <c r="C80" s="26"/>
-      <c r="D80" s="27"/>
-      <c r="E80" s="27"/>
-      <c r="F80" s="26"/>
-      <c r="G80" s="26"/>
-      <c r="H80" s="26"/>
-      <c r="O80" s="26"/>
-      <c r="P80" s="27"/>
-      <c r="Q80" s="27"/>
-      <c r="R80" s="26"/>
-      <c r="S80" s="26"/>
-      <c r="T80" s="26"/>
-      <c r="AH80"/>
-      <c r="AI80"/>
       <c r="AJ80"/>
       <c r="AK80"/>
       <c r="AL80"/>
@@ -6027,26 +6123,9 @@
       <c r="AP80"/>
       <c r="AQ80"/>
       <c r="AR80"/>
-      <c r="AT80" s="40"/>
-    </row>
-    <row r="81" spans="2:47" ht="117" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B81" s="25"/>
-      <c r="C81" s="38" t="s">
-        <v>10</v>
-      </c>
-      <c r="D81" s="39"/>
-      <c r="E81" s="39"/>
-      <c r="F81" s="39"/>
-      <c r="G81" s="39"/>
-      <c r="H81" s="39"/>
-      <c r="O81" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="P81" s="39"/>
-      <c r="Q81" s="39"/>
-      <c r="R81" s="39"/>
-      <c r="S81" s="39"/>
-      <c r="T81" s="39"/>
+      <c r="AT80" s="39"/>
+    </row>
+    <row r="81" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AH81"/>
       <c r="AI81"/>
       <c r="AJ81"/>
@@ -6058,9 +6137,21 @@
       <c r="AP81"/>
       <c r="AQ81"/>
       <c r="AR81"/>
-      <c r="AT81" s="40"/>
+      <c r="AT81" s="39"/>
     </row>
     <row r="82" spans="2:47" x14ac:dyDescent="0.2">
+      <c r="C82" s="26"/>
+      <c r="D82" s="27"/>
+      <c r="E82" s="27"/>
+      <c r="F82" s="26"/>
+      <c r="G82" s="26"/>
+      <c r="H82" s="26"/>
+      <c r="O82" s="26"/>
+      <c r="P82" s="27"/>
+      <c r="Q82" s="27"/>
+      <c r="R82" s="26"/>
+      <c r="S82" s="26"/>
+      <c r="T82" s="26"/>
       <c r="AH82"/>
       <c r="AI82"/>
       <c r="AJ82"/>
@@ -6072,9 +6163,26 @@
       <c r="AP82"/>
       <c r="AQ82"/>
       <c r="AR82"/>
-      <c r="AT82" s="40"/>
-    </row>
-    <row r="83" spans="2:47" x14ac:dyDescent="0.2">
+      <c r="AT82" s="39"/>
+    </row>
+    <row r="83" spans="2:47" ht="117" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B83" s="25"/>
+      <c r="C83" s="37" t="s">
+        <v>10</v>
+      </c>
+      <c r="D83" s="38"/>
+      <c r="E83" s="38"/>
+      <c r="F83" s="38"/>
+      <c r="G83" s="38"/>
+      <c r="H83" s="38"/>
+      <c r="O83" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="P83" s="38"/>
+      <c r="Q83" s="38"/>
+      <c r="R83" s="38"/>
+      <c r="S83" s="38"/>
+      <c r="T83" s="38"/>
       <c r="AH83"/>
       <c r="AI83"/>
       <c r="AJ83"/>
@@ -6086,7 +6194,7 @@
       <c r="AP83"/>
       <c r="AQ83"/>
       <c r="AR83"/>
-      <c r="AT83" s="40"/>
+      <c r="AT83" s="39"/>
     </row>
     <row r="84" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AH84"/>
@@ -6100,7 +6208,7 @@
       <c r="AP84"/>
       <c r="AQ84"/>
       <c r="AR84"/>
-      <c r="AT84" s="40"/>
+      <c r="AT84" s="39"/>
     </row>
     <row r="85" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AH85"/>
@@ -6114,62 +6222,82 @@
       <c r="AP85"/>
       <c r="AQ85"/>
       <c r="AR85"/>
-      <c r="AT85" s="40"/>
+      <c r="AT85" s="39"/>
     </row>
     <row r="86" spans="2:47" x14ac:dyDescent="0.2">
-      <c r="AS86" s="2"/>
-      <c r="AT86" s="41"/>
+      <c r="AH86"/>
+      <c r="AI86"/>
+      <c r="AJ86"/>
+      <c r="AK86"/>
+      <c r="AL86"/>
+      <c r="AM86"/>
+      <c r="AN86"/>
+      <c r="AO86"/>
+      <c r="AP86"/>
+      <c r="AQ86"/>
+      <c r="AR86"/>
+      <c r="AT86" s="39"/>
     </row>
     <row r="87" spans="2:47" x14ac:dyDescent="0.2">
-      <c r="AS87" s="2"/>
-      <c r="AT87" s="41"/>
+      <c r="AH87"/>
+      <c r="AI87"/>
+      <c r="AJ87"/>
+      <c r="AK87"/>
+      <c r="AL87"/>
+      <c r="AM87"/>
+      <c r="AN87"/>
+      <c r="AO87"/>
+      <c r="AP87"/>
+      <c r="AQ87"/>
+      <c r="AR87"/>
+      <c r="AT87" s="39"/>
     </row>
     <row r="88" spans="2:47" x14ac:dyDescent="0.2">
-      <c r="D88" s="2"/>
-      <c r="E88" s="2"/>
       <c r="AS88" s="2"/>
-      <c r="AT88" s="41"/>
+      <c r="AT88" s="40"/>
     </row>
     <row r="89" spans="2:47" x14ac:dyDescent="0.2">
-      <c r="D89" s="2"/>
-      <c r="E89" s="2"/>
-      <c r="AS89" s="44"/>
-      <c r="AT89" s="43"/>
+      <c r="AS89" s="2"/>
+      <c r="AT89" s="40"/>
     </row>
     <row r="90" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D90" s="2"/>
       <c r="E90" s="2"/>
-      <c r="AS90" s="44"/>
-      <c r="AU90"/>
-    </row>
-    <row r="91" spans="2:47" s="42" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="AS91" s="45"/>
-      <c r="AT91"/>
-      <c r="AU91"/>
+      <c r="AS90" s="2"/>
+      <c r="AT90" s="40"/>
+    </row>
+    <row r="91" spans="2:47" x14ac:dyDescent="0.2">
+      <c r="D91" s="2"/>
+      <c r="E91" s="2"/>
+      <c r="AS91" s="43"/>
+      <c r="AT91" s="42"/>
     </row>
     <row r="92" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D92" s="2"/>
       <c r="E92" s="2"/>
-      <c r="AS92" s="2"/>
+      <c r="AS92" s="43"/>
       <c r="AU92"/>
     </row>
-    <row r="93" spans="2:47" x14ac:dyDescent="0.2">
-      <c r="D93" s="2"/>
-      <c r="E93" s="2"/>
+    <row r="93" spans="2:47" s="41" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AS93" s="44"/>
+      <c r="AT93"/>
+      <c r="AU93"/>
     </row>
     <row r="94" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D94" s="2"/>
       <c r="E94" s="2"/>
+      <c r="AS94" s="2"/>
+      <c r="AU94"/>
     </row>
     <row r="95" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D95" s="2"/>
       <c r="E95" s="2"/>
     </row>
-    <row r="96" spans="2:47" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D96" s="2"/>
       <c r="E96" s="2"/>
     </row>
-    <row r="97" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D97" s="2"/>
       <c r="E97" s="2"/>
     </row>
@@ -6389,11 +6517,22 @@
       <c r="D151" s="2"/>
       <c r="E151" s="2"/>
     </row>
+    <row r="152" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="D152" s="2"/>
+      <c r="E152" s="2"/>
+    </row>
+    <row r="153" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
+      <c r="D153" s="2"/>
+      <c r="E153" s="2"/>
+    </row>
+    <row r="154" spans="4:5" x14ac:dyDescent="0.2"/>
+    <row r="155" spans="4:5" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="C81:H81"/>
-    <mergeCell ref="O81:T81"/>
-    <mergeCell ref="C8:T8"/>
+  <mergeCells count="4">
+    <mergeCell ref="C83:H83"/>
+    <mergeCell ref="O83:T83"/>
+    <mergeCell ref="C8:T10"/>
+    <mergeCell ref="C19:T19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
created plot in notebook
</commit_message>
<xml_diff>
--- a/Template_Build_survival_curve_hazard_ratio_20260420_DZ.xlsx
+++ b/Template_Build_survival_curve_hazard_ratio_20260420_DZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xinzhao/DS_Projects/build-survival-curve-hazardratio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{837BF602-9530-8149-AE74-E571DF189102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B26BAF6-BC65-F04E-842E-24CB3425B85D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="600" windowWidth="37220" windowHeight="21000" xr2:uid="{120A936B-BDCD-7149-9B97-5E03885B164C}"/>
   </bookViews>
@@ -155,7 +155,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -416,7 +416,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -524,20 +524,11 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -549,14 +540,17 @@
     <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3067,7 +3061,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A3DAE5-C576-0C46-AA24-CA8BC1EAE5FA}">
   <dimension ref="A1:AU155"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="16" zeroHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="16" zeroHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="10.83203125" style="2" customWidth="1"/>
     <col min="3" max="3" width="19.83203125" style="2" customWidth="1"/>
@@ -3082,16 +3076,16 @@
     <col min="48" max="16384" width="10.83203125" style="2" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:47" s="8" customFormat="1" ht="140" customHeight="1">
+    <row r="1" spans="2:47" s="8" customFormat="1" ht="140" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
-      <c r="K1" s="45" t="s">
+      <c r="K1" s="42" t="s">
         <v>16</v>
       </c>
       <c r="AT1"/>
       <c r="AU1"/>
     </row>
-    <row r="2" spans="2:47">
+    <row r="2" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AH2"/>
       <c r="AI2"/>
       <c r="AJ2"/>
@@ -3103,9 +3097,9 @@
       <c r="AP2"/>
       <c r="AQ2"/>
       <c r="AR2"/>
-      <c r="AT2" s="39"/>
-    </row>
-    <row r="3" spans="2:47">
+      <c r="AT2" s="37"/>
+    </row>
+    <row r="3" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AH3"/>
       <c r="AI3"/>
       <c r="AJ3"/>
@@ -3117,9 +3111,9 @@
       <c r="AP3"/>
       <c r="AQ3"/>
       <c r="AR3"/>
-      <c r="AT3" s="39"/>
-    </row>
-    <row r="4" spans="2:47" ht="24">
+      <c r="AT3" s="37"/>
+    </row>
+    <row r="4" spans="2:47" ht="24" x14ac:dyDescent="0.2">
       <c r="C4" s="28"/>
       <c r="D4" s="29"/>
       <c r="E4" s="29"/>
@@ -3151,10 +3145,10 @@
       <c r="AP4"/>
       <c r="AQ4"/>
       <c r="AR4"/>
-      <c r="AT4" s="39"/>
-    </row>
-    <row r="5" spans="2:47" ht="28" thickBot="1">
-      <c r="B5" s="48" t="s">
+      <c r="AT4" s="37"/>
+    </row>
+    <row r="5" spans="2:47" ht="28" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="44" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="32"/>
@@ -3199,9 +3193,9 @@
       <c r="AP5"/>
       <c r="AQ5"/>
       <c r="AR5"/>
-      <c r="AT5" s="39"/>
-    </row>
-    <row r="6" spans="2:47" ht="28" thickTop="1">
+      <c r="AT5" s="37"/>
+    </row>
+    <row r="6" spans="2:47" ht="28" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B6" s="31"/>
       <c r="C6" s="34"/>
       <c r="D6" s="35"/>
@@ -3234,43 +3228,42 @@
       <c r="AP6"/>
       <c r="AQ6"/>
       <c r="AR6"/>
-      <c r="AT6" s="39"/>
-    </row>
-    <row r="7" spans="2:47" ht="343" customHeight="1">
+      <c r="AT6" s="37"/>
+    </row>
+    <row r="7" spans="2:47" ht="343" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="31"/>
-      <c r="C7" s="49" t="s">
+      <c r="C7" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="49"/>
-      <c r="I7" s="49"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="49"/>
-      <c r="L7" s="49"/>
-      <c r="M7" s="49"/>
-      <c r="N7" s="49"/>
-      <c r="O7" s="49"/>
-      <c r="P7" s="49"/>
-      <c r="Q7" s="49"/>
-      <c r="R7" s="49"/>
-      <c r="S7" s="49"/>
-      <c r="T7" s="49"/>
-      <c r="U7" s="46"/>
-      <c r="V7" s="46"/>
-      <c r="W7" s="46"/>
-      <c r="X7" s="46"/>
-      <c r="Y7" s="46"/>
-      <c r="Z7" s="46"/>
-      <c r="AA7" s="46"/>
-      <c r="AB7" s="46"/>
-      <c r="AC7" s="46"/>
-      <c r="AD7" s="46"/>
-      <c r="AE7" s="46"/>
-      <c r="AF7" s="46"/>
-      <c r="AG7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47"/>
+      <c r="L7" s="47"/>
+      <c r="M7" s="47"/>
+      <c r="N7" s="47"/>
+      <c r="O7" s="47"/>
+      <c r="P7" s="47"/>
+      <c r="Q7" s="47"/>
+      <c r="R7" s="47"/>
+      <c r="S7" s="47"/>
+      <c r="T7" s="47"/>
+      <c r="U7" s="43"/>
+      <c r="V7" s="43"/>
+      <c r="W7" s="43"/>
+      <c r="X7" s="43"/>
+      <c r="Y7" s="43"/>
+      <c r="Z7" s="43"/>
+      <c r="AA7" s="43"/>
+      <c r="AB7" s="43"/>
+      <c r="AC7" s="43"/>
+      <c r="AD7" s="43"/>
+      <c r="AE7" s="43"/>
+      <c r="AF7" s="43"/>
       <c r="AH7"/>
       <c r="AI7"/>
       <c r="AJ7"/>
@@ -3282,9 +3275,9 @@
       <c r="AP7"/>
       <c r="AQ7"/>
       <c r="AR7"/>
-      <c r="AT7" s="39"/>
-    </row>
-    <row r="8" spans="2:47" ht="27">
+      <c r="AT7" s="37"/>
+    </row>
+    <row r="8" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B8" s="31"/>
       <c r="C8"/>
       <c r="D8"/>
@@ -3317,9 +3310,9 @@
       <c r="AP8"/>
       <c r="AQ8"/>
       <c r="AR8"/>
-      <c r="AT8" s="39"/>
-    </row>
-    <row r="9" spans="2:47" ht="27">
+      <c r="AT8" s="37"/>
+    </row>
+    <row r="9" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B9" s="31"/>
       <c r="C9"/>
       <c r="D9"/>
@@ -3352,9 +3345,9 @@
       <c r="AP9"/>
       <c r="AQ9"/>
       <c r="AR9"/>
-      <c r="AT9" s="39"/>
-    </row>
-    <row r="10" spans="2:47" ht="27">
+      <c r="AT9" s="37"/>
+    </row>
+    <row r="10" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B10" s="31"/>
       <c r="C10" s="34"/>
       <c r="D10" s="35"/>
@@ -3387,9 +3380,9 @@
       <c r="AP10"/>
       <c r="AQ10"/>
       <c r="AR10"/>
-      <c r="AT10" s="39"/>
-    </row>
-    <row r="11" spans="2:47" ht="27">
+      <c r="AT10" s="37"/>
+    </row>
+    <row r="11" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B11" s="31"/>
       <c r="C11" s="34"/>
       <c r="D11" s="35"/>
@@ -3422,9 +3415,9 @@
       <c r="AP11"/>
       <c r="AQ11"/>
       <c r="AR11"/>
-      <c r="AT11" s="39"/>
-    </row>
-    <row r="12" spans="2:47" ht="27">
+      <c r="AT11" s="37"/>
+    </row>
+    <row r="12" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B12" s="31"/>
       <c r="C12" s="34"/>
       <c r="D12" s="35"/>
@@ -3457,9 +3450,9 @@
       <c r="AP12"/>
       <c r="AQ12"/>
       <c r="AR12"/>
-      <c r="AT12" s="39"/>
-    </row>
-    <row r="13" spans="2:47" ht="27">
+      <c r="AT12" s="37"/>
+    </row>
+    <row r="13" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B13" s="31"/>
       <c r="C13" s="34"/>
       <c r="D13" s="35"/>
@@ -3492,9 +3485,9 @@
       <c r="AP13"/>
       <c r="AQ13"/>
       <c r="AR13"/>
-      <c r="AT13" s="39"/>
-    </row>
-    <row r="14" spans="2:47" ht="27">
+      <c r="AT13" s="37"/>
+    </row>
+    <row r="14" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B14" s="31"/>
       <c r="C14" s="34"/>
       <c r="D14" s="35"/>
@@ -3527,9 +3520,9 @@
       <c r="AP14"/>
       <c r="AQ14"/>
       <c r="AR14"/>
-      <c r="AT14" s="39"/>
-    </row>
-    <row r="15" spans="2:47" ht="27">
+      <c r="AT14" s="37"/>
+    </row>
+    <row r="15" spans="2:47" ht="27" x14ac:dyDescent="0.2">
       <c r="B15" s="31"/>
       <c r="C15" s="34"/>
       <c r="D15" s="35"/>
@@ -3562,9 +3555,9 @@
       <c r="AP15"/>
       <c r="AQ15"/>
       <c r="AR15"/>
-      <c r="AT15" s="39"/>
-    </row>
-    <row r="16" spans="2:47" ht="28" thickBot="1">
+      <c r="AT15" s="37"/>
+    </row>
+    <row r="16" spans="2:47" ht="28" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B16" s="36" t="s">
         <v>4</v>
       </c>
@@ -3610,9 +3603,9 @@
       <c r="AP16"/>
       <c r="AQ16"/>
       <c r="AR16"/>
-      <c r="AT16" s="39"/>
-    </row>
-    <row r="17" spans="2:46" ht="28" thickTop="1">
+      <c r="AT16" s="37"/>
+    </row>
+    <row r="17" spans="2:46" ht="28" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B17" s="31"/>
       <c r="C17" s="34"/>
       <c r="D17" s="35"/>
@@ -3645,30 +3638,30 @@
       <c r="AP17"/>
       <c r="AQ17"/>
       <c r="AR17"/>
-      <c r="AT17" s="39"/>
-    </row>
-    <row r="18" spans="2:46" ht="91" customHeight="1">
+      <c r="AT17" s="37"/>
+    </row>
+    <row r="18" spans="2:46" ht="91" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="31"/>
-      <c r="C18" s="50" t="s">
+      <c r="C18" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="50"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
-      <c r="I18" s="50"/>
-      <c r="J18" s="50"/>
-      <c r="K18" s="50"/>
-      <c r="L18" s="50"/>
-      <c r="M18" s="50"/>
-      <c r="N18" s="50"/>
-      <c r="O18" s="50"/>
-      <c r="P18" s="50"/>
-      <c r="Q18" s="50"/>
-      <c r="R18" s="50"/>
-      <c r="S18" s="50"/>
-      <c r="T18" s="50"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="48"/>
+      <c r="G18" s="48"/>
+      <c r="H18" s="48"/>
+      <c r="I18" s="48"/>
+      <c r="J18" s="48"/>
+      <c r="K18" s="48"/>
+      <c r="L18" s="48"/>
+      <c r="M18" s="48"/>
+      <c r="N18" s="48"/>
+      <c r="O18" s="48"/>
+      <c r="P18" s="48"/>
+      <c r="Q18" s="48"/>
+      <c r="R18" s="48"/>
+      <c r="S18" s="48"/>
+      <c r="T18" s="48"/>
       <c r="U18" s="28"/>
       <c r="V18" s="28"/>
       <c r="AH18"/>
@@ -3682,9 +3675,9 @@
       <c r="AP18"/>
       <c r="AQ18"/>
       <c r="AR18"/>
-      <c r="AT18" s="39"/>
-    </row>
-    <row r="19" spans="2:46" ht="27">
+      <c r="AT18" s="37"/>
+    </row>
+    <row r="19" spans="2:46" ht="27" x14ac:dyDescent="0.2">
       <c r="B19" s="31"/>
       <c r="C19" s="34"/>
       <c r="D19" s="35"/>
@@ -3717,9 +3710,9 @@
       <c r="AP19"/>
       <c r="AQ19"/>
       <c r="AR19"/>
-      <c r="AT19" s="39"/>
-    </row>
-    <row r="20" spans="2:46" ht="27">
+      <c r="AT19" s="37"/>
+    </row>
+    <row r="20" spans="2:46" ht="27" x14ac:dyDescent="0.2">
       <c r="B20" s="31"/>
       <c r="C20" s="34"/>
       <c r="D20" s="35"/>
@@ -3752,9 +3745,9 @@
       <c r="AP20"/>
       <c r="AQ20"/>
       <c r="AR20"/>
-      <c r="AT20" s="39"/>
-    </row>
-    <row r="21" spans="2:46" ht="28" thickBot="1">
+      <c r="AT20" s="37"/>
+    </row>
+    <row r="21" spans="2:46" ht="28" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B21" s="31"/>
       <c r="C21" s="36" t="s">
         <v>3</v>
@@ -3802,9 +3795,9 @@
       <c r="AP21"/>
       <c r="AQ21"/>
       <c r="AR21"/>
-      <c r="AT21" s="39"/>
-    </row>
-    <row r="22" spans="2:46" ht="17" thickTop="1">
+      <c r="AT21" s="37"/>
+    </row>
+    <row r="22" spans="2:46" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="AJ22"/>
       <c r="AK22"/>
       <c r="AL22"/>
@@ -3814,9 +3807,9 @@
       <c r="AP22"/>
       <c r="AQ22"/>
       <c r="AR22"/>
-      <c r="AT22" s="39"/>
-    </row>
-    <row r="23" spans="2:46">
+      <c r="AT22" s="37"/>
+    </row>
+    <row r="23" spans="2:46" x14ac:dyDescent="0.2">
       <c r="AJ23"/>
       <c r="AK23"/>
       <c r="AL23"/>
@@ -3826,9 +3819,9 @@
       <c r="AP23"/>
       <c r="AQ23"/>
       <c r="AR23"/>
-      <c r="AT23" s="39"/>
-    </row>
-    <row r="24" spans="2:46">
+      <c r="AT23" s="37"/>
+    </row>
+    <row r="24" spans="2:46" x14ac:dyDescent="0.2">
       <c r="AJ24"/>
       <c r="AK24"/>
       <c r="AL24"/>
@@ -3838,9 +3831,9 @@
       <c r="AP24"/>
       <c r="AQ24"/>
       <c r="AR24"/>
-      <c r="AT24" s="39"/>
-    </row>
-    <row r="25" spans="2:46" s="4" customFormat="1" ht="24">
+      <c r="AT24" s="37"/>
+    </row>
+    <row r="25" spans="2:46" s="4" customFormat="1" ht="24" x14ac:dyDescent="0.2">
       <c r="C25" s="5" t="s">
         <v>7</v>
       </c>
@@ -3878,9 +3871,9 @@
       <c r="AQ25"/>
       <c r="AR25"/>
       <c r="AS25"/>
-      <c r="AT25" s="39"/>
-    </row>
-    <row r="26" spans="2:46">
+      <c r="AT25" s="37"/>
+    </row>
+    <row r="26" spans="2:46" x14ac:dyDescent="0.2">
       <c r="AJ26"/>
       <c r="AK26"/>
       <c r="AL26"/>
@@ -3890,9 +3883,9 @@
       <c r="AP26"/>
       <c r="AQ26"/>
       <c r="AR26"/>
-      <c r="AT26" s="39"/>
-    </row>
-    <row r="27" spans="2:46" s="1" customFormat="1" ht="44" customHeight="1" thickBot="1">
+      <c r="AT26" s="37"/>
+    </row>
+    <row r="27" spans="2:46" s="1" customFormat="1" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C27" s="13" t="s">
         <v>5</v>
       </c>
@@ -3931,9 +3924,9 @@
       <c r="AQ27"/>
       <c r="AR27"/>
       <c r="AS27"/>
-      <c r="AT27" s="39"/>
-    </row>
-    <row r="28" spans="2:46">
+      <c r="AT27" s="37"/>
+    </row>
+    <row r="28" spans="2:46" x14ac:dyDescent="0.2">
       <c r="C28" s="19">
         <v>0</v>
       </c>
@@ -3976,9 +3969,9 @@
       <c r="AP28"/>
       <c r="AQ28"/>
       <c r="AR28"/>
-      <c r="AT28" s="39"/>
-    </row>
-    <row r="29" spans="2:46">
+      <c r="AT28" s="37"/>
+    </row>
+    <row r="29" spans="2:46" x14ac:dyDescent="0.2">
       <c r="C29" s="20">
         <v>1</v>
       </c>
@@ -4018,9 +4011,9 @@
       <c r="AP29"/>
       <c r="AQ29"/>
       <c r="AR29"/>
-      <c r="AT29" s="39"/>
-    </row>
-    <row r="30" spans="2:46">
+      <c r="AT29" s="37"/>
+    </row>
+    <row r="30" spans="2:46" x14ac:dyDescent="0.2">
       <c r="C30" s="20">
         <v>2</v>
       </c>
@@ -4060,9 +4053,9 @@
       <c r="AP30"/>
       <c r="AQ30"/>
       <c r="AR30"/>
-      <c r="AT30" s="39"/>
-    </row>
-    <row r="31" spans="2:46">
+      <c r="AT30" s="37"/>
+    </row>
+    <row r="31" spans="2:46" x14ac:dyDescent="0.2">
       <c r="C31" s="20">
         <v>3</v>
       </c>
@@ -4102,9 +4095,9 @@
       <c r="AP31"/>
       <c r="AQ31"/>
       <c r="AR31"/>
-      <c r="AT31" s="39"/>
-    </row>
-    <row r="32" spans="2:46">
+      <c r="AT31" s="37"/>
+    </row>
+    <row r="32" spans="2:46" x14ac:dyDescent="0.2">
       <c r="C32" s="20">
         <v>4</v>
       </c>
@@ -4144,9 +4137,9 @@
       <c r="AP32"/>
       <c r="AQ32"/>
       <c r="AR32"/>
-      <c r="AT32" s="39"/>
-    </row>
-    <row r="33" spans="3:46">
+      <c r="AT32" s="37"/>
+    </row>
+    <row r="33" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C33" s="20">
         <v>5</v>
       </c>
@@ -4186,9 +4179,9 @@
       <c r="AP33"/>
       <c r="AQ33"/>
       <c r="AR33"/>
-      <c r="AT33" s="39"/>
-    </row>
-    <row r="34" spans="3:46">
+      <c r="AT33" s="37"/>
+    </row>
+    <row r="34" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C34" s="20">
         <v>6</v>
       </c>
@@ -4228,9 +4221,9 @@
       <c r="AP34"/>
       <c r="AQ34"/>
       <c r="AR34"/>
-      <c r="AT34" s="39"/>
-    </row>
-    <row r="35" spans="3:46">
+      <c r="AT34" s="37"/>
+    </row>
+    <row r="35" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C35" s="20">
         <v>7</v>
       </c>
@@ -4270,9 +4263,9 @@
       <c r="AP35"/>
       <c r="AQ35"/>
       <c r="AR35"/>
-      <c r="AT35" s="39"/>
-    </row>
-    <row r="36" spans="3:46">
+      <c r="AT35" s="37"/>
+    </row>
+    <row r="36" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C36" s="20">
         <v>8</v>
       </c>
@@ -4312,9 +4305,9 @@
       <c r="AP36"/>
       <c r="AQ36"/>
       <c r="AR36"/>
-      <c r="AT36" s="39"/>
-    </row>
-    <row r="37" spans="3:46">
+      <c r="AT36" s="37"/>
+    </row>
+    <row r="37" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C37" s="20">
         <v>9</v>
       </c>
@@ -4354,9 +4347,9 @@
       <c r="AP37"/>
       <c r="AQ37"/>
       <c r="AR37"/>
-      <c r="AT37" s="39"/>
-    </row>
-    <row r="38" spans="3:46">
+      <c r="AT37" s="37"/>
+    </row>
+    <row r="38" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C38" s="20">
         <v>10</v>
       </c>
@@ -4396,9 +4389,9 @@
       <c r="AP38"/>
       <c r="AQ38"/>
       <c r="AR38"/>
-      <c r="AT38" s="39"/>
-    </row>
-    <row r="39" spans="3:46">
+      <c r="AT38" s="37"/>
+    </row>
+    <row r="39" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C39" s="20">
         <v>11</v>
       </c>
@@ -4438,9 +4431,9 @@
       <c r="AP39"/>
       <c r="AQ39"/>
       <c r="AR39"/>
-      <c r="AT39" s="39"/>
-    </row>
-    <row r="40" spans="3:46">
+      <c r="AT39" s="37"/>
+    </row>
+    <row r="40" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C40" s="20">
         <v>12</v>
       </c>
@@ -4480,9 +4473,9 @@
       <c r="AP40"/>
       <c r="AQ40"/>
       <c r="AR40"/>
-      <c r="AT40" s="39"/>
-    </row>
-    <row r="41" spans="3:46">
+      <c r="AT40" s="37"/>
+    </row>
+    <row r="41" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C41" s="20">
         <v>13</v>
       </c>
@@ -4522,9 +4515,9 @@
       <c r="AP41"/>
       <c r="AQ41"/>
       <c r="AR41"/>
-      <c r="AT41" s="39"/>
-    </row>
-    <row r="42" spans="3:46">
+      <c r="AT41" s="37"/>
+    </row>
+    <row r="42" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C42" s="20">
         <v>14</v>
       </c>
@@ -4564,9 +4557,9 @@
       <c r="AP42"/>
       <c r="AQ42"/>
       <c r="AR42"/>
-      <c r="AT42" s="39"/>
-    </row>
-    <row r="43" spans="3:46">
+      <c r="AT42" s="37"/>
+    </row>
+    <row r="43" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C43" s="20">
         <v>15</v>
       </c>
@@ -4606,9 +4599,9 @@
       <c r="AP43"/>
       <c r="AQ43"/>
       <c r="AR43"/>
-      <c r="AT43" s="39"/>
-    </row>
-    <row r="44" spans="3:46">
+      <c r="AT43" s="37"/>
+    </row>
+    <row r="44" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C44" s="20">
         <v>16</v>
       </c>
@@ -4648,9 +4641,9 @@
       <c r="AP44"/>
       <c r="AQ44"/>
       <c r="AR44"/>
-      <c r="AT44" s="39"/>
-    </row>
-    <row r="45" spans="3:46">
+      <c r="AT44" s="37"/>
+    </row>
+    <row r="45" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C45" s="20">
         <v>17</v>
       </c>
@@ -4690,9 +4683,9 @@
       <c r="AP45"/>
       <c r="AQ45"/>
       <c r="AR45"/>
-      <c r="AT45" s="39"/>
-    </row>
-    <row r="46" spans="3:46">
+      <c r="AT45" s="37"/>
+    </row>
+    <row r="46" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C46" s="20">
         <v>18</v>
       </c>
@@ -4732,9 +4725,9 @@
       <c r="AP46"/>
       <c r="AQ46"/>
       <c r="AR46"/>
-      <c r="AT46" s="39"/>
-    </row>
-    <row r="47" spans="3:46">
+      <c r="AT46" s="37"/>
+    </row>
+    <row r="47" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C47" s="20">
         <v>19</v>
       </c>
@@ -4774,9 +4767,9 @@
       <c r="AP47"/>
       <c r="AQ47"/>
       <c r="AR47"/>
-      <c r="AT47" s="39"/>
-    </row>
-    <row r="48" spans="3:46">
+      <c r="AT47" s="37"/>
+    </row>
+    <row r="48" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C48" s="20">
         <v>20</v>
       </c>
@@ -4816,9 +4809,9 @@
       <c r="AP48"/>
       <c r="AQ48"/>
       <c r="AR48"/>
-      <c r="AT48" s="39"/>
-    </row>
-    <row r="49" spans="3:46">
+      <c r="AT48" s="37"/>
+    </row>
+    <row r="49" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C49" s="20">
         <v>21</v>
       </c>
@@ -4858,9 +4851,9 @@
       <c r="AP49"/>
       <c r="AQ49"/>
       <c r="AR49"/>
-      <c r="AT49" s="39"/>
-    </row>
-    <row r="50" spans="3:46">
+      <c r="AT49" s="37"/>
+    </row>
+    <row r="50" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C50" s="20">
         <v>22</v>
       </c>
@@ -4900,9 +4893,9 @@
       <c r="AP50"/>
       <c r="AQ50"/>
       <c r="AR50"/>
-      <c r="AT50" s="39"/>
-    </row>
-    <row r="51" spans="3:46">
+      <c r="AT50" s="37"/>
+    </row>
+    <row r="51" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C51" s="20">
         <v>23</v>
       </c>
@@ -4942,9 +4935,9 @@
       <c r="AP51"/>
       <c r="AQ51"/>
       <c r="AR51"/>
-      <c r="AT51" s="39"/>
-    </row>
-    <row r="52" spans="3:46">
+      <c r="AT51" s="37"/>
+    </row>
+    <row r="52" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C52" s="20">
         <v>24</v>
       </c>
@@ -4984,9 +4977,9 @@
       <c r="AP52"/>
       <c r="AQ52"/>
       <c r="AR52"/>
-      <c r="AT52" s="39"/>
-    </row>
-    <row r="53" spans="3:46">
+      <c r="AT52" s="37"/>
+    </row>
+    <row r="53" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C53" s="20">
         <v>25</v>
       </c>
@@ -5026,9 +5019,9 @@
       <c r="AP53"/>
       <c r="AQ53"/>
       <c r="AR53"/>
-      <c r="AT53" s="39"/>
-    </row>
-    <row r="54" spans="3:46">
+      <c r="AT53" s="37"/>
+    </row>
+    <row r="54" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C54" s="20">
         <v>26</v>
       </c>
@@ -5068,9 +5061,9 @@
       <c r="AP54"/>
       <c r="AQ54"/>
       <c r="AR54"/>
-      <c r="AT54" s="39"/>
-    </row>
-    <row r="55" spans="3:46">
+      <c r="AT54" s="37"/>
+    </row>
+    <row r="55" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C55" s="20">
         <v>27</v>
       </c>
@@ -5110,9 +5103,9 @@
       <c r="AP55"/>
       <c r="AQ55"/>
       <c r="AR55"/>
-      <c r="AT55" s="39"/>
-    </row>
-    <row r="56" spans="3:46">
+      <c r="AT55" s="37"/>
+    </row>
+    <row r="56" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C56" s="20">
         <v>28</v>
       </c>
@@ -5152,9 +5145,9 @@
       <c r="AP56"/>
       <c r="AQ56"/>
       <c r="AR56"/>
-      <c r="AT56" s="39"/>
-    </row>
-    <row r="57" spans="3:46">
+      <c r="AT56" s="37"/>
+    </row>
+    <row r="57" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C57" s="20">
         <v>29</v>
       </c>
@@ -5194,9 +5187,9 @@
       <c r="AP57"/>
       <c r="AQ57"/>
       <c r="AR57"/>
-      <c r="AT57" s="39"/>
-    </row>
-    <row r="58" spans="3:46">
+      <c r="AT57" s="37"/>
+    </row>
+    <row r="58" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C58" s="20">
         <v>30</v>
       </c>
@@ -5236,9 +5229,9 @@
       <c r="AP58"/>
       <c r="AQ58"/>
       <c r="AR58"/>
-      <c r="AT58" s="39"/>
-    </row>
-    <row r="59" spans="3:46">
+      <c r="AT58" s="37"/>
+    </row>
+    <row r="59" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C59" s="20">
         <v>31</v>
       </c>
@@ -5278,9 +5271,9 @@
       <c r="AP59"/>
       <c r="AQ59"/>
       <c r="AR59"/>
-      <c r="AT59" s="39"/>
-    </row>
-    <row r="60" spans="3:46">
+      <c r="AT59" s="37"/>
+    </row>
+    <row r="60" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C60" s="20">
         <v>32</v>
       </c>
@@ -5320,9 +5313,9 @@
       <c r="AP60"/>
       <c r="AQ60"/>
       <c r="AR60"/>
-      <c r="AT60" s="39"/>
-    </row>
-    <row r="61" spans="3:46">
+      <c r="AT60" s="37"/>
+    </row>
+    <row r="61" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C61" s="20">
         <v>33</v>
       </c>
@@ -5362,9 +5355,9 @@
       <c r="AP61"/>
       <c r="AQ61"/>
       <c r="AR61"/>
-      <c r="AT61" s="39"/>
-    </row>
-    <row r="62" spans="3:46">
+      <c r="AT61" s="37"/>
+    </row>
+    <row r="62" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C62" s="20">
         <v>34</v>
       </c>
@@ -5404,9 +5397,9 @@
       <c r="AP62"/>
       <c r="AQ62"/>
       <c r="AR62"/>
-      <c r="AT62" s="39"/>
-    </row>
-    <row r="63" spans="3:46">
+      <c r="AT62" s="37"/>
+    </row>
+    <row r="63" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C63" s="20">
         <v>35</v>
       </c>
@@ -5446,9 +5439,9 @@
       <c r="AP63"/>
       <c r="AQ63"/>
       <c r="AR63"/>
-      <c r="AT63" s="39"/>
-    </row>
-    <row r="64" spans="3:46">
+      <c r="AT63" s="37"/>
+    </row>
+    <row r="64" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C64" s="20">
         <v>36</v>
       </c>
@@ -5488,9 +5481,9 @@
       <c r="AP64"/>
       <c r="AQ64"/>
       <c r="AR64"/>
-      <c r="AT64" s="39"/>
-    </row>
-    <row r="65" spans="3:46">
+      <c r="AT64" s="37"/>
+    </row>
+    <row r="65" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C65" s="20">
         <v>37</v>
       </c>
@@ -5530,9 +5523,9 @@
       <c r="AP65"/>
       <c r="AQ65"/>
       <c r="AR65"/>
-      <c r="AT65" s="39"/>
-    </row>
-    <row r="66" spans="3:46">
+      <c r="AT65" s="37"/>
+    </row>
+    <row r="66" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C66" s="20">
         <v>38</v>
       </c>
@@ -5572,9 +5565,9 @@
       <c r="AP66"/>
       <c r="AQ66"/>
       <c r="AR66"/>
-      <c r="AT66" s="39"/>
-    </row>
-    <row r="67" spans="3:46">
+      <c r="AT66" s="37"/>
+    </row>
+    <row r="67" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C67" s="20">
         <v>39</v>
       </c>
@@ -5614,9 +5607,9 @@
       <c r="AP67"/>
       <c r="AQ67"/>
       <c r="AR67"/>
-      <c r="AT67" s="39"/>
-    </row>
-    <row r="68" spans="3:46">
+      <c r="AT67" s="37"/>
+    </row>
+    <row r="68" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C68" s="20">
         <v>40</v>
       </c>
@@ -5656,9 +5649,9 @@
       <c r="AP68"/>
       <c r="AQ68"/>
       <c r="AR68"/>
-      <c r="AT68" s="39"/>
-    </row>
-    <row r="69" spans="3:46">
+      <c r="AT68" s="37"/>
+    </row>
+    <row r="69" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C69" s="20">
         <v>41</v>
       </c>
@@ -5698,9 +5691,9 @@
       <c r="AP69"/>
       <c r="AQ69"/>
       <c r="AR69"/>
-      <c r="AT69" s="39"/>
-    </row>
-    <row r="70" spans="3:46">
+      <c r="AT69" s="37"/>
+    </row>
+    <row r="70" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C70" s="20">
         <v>42</v>
       </c>
@@ -5740,9 +5733,9 @@
       <c r="AP70"/>
       <c r="AQ70"/>
       <c r="AR70"/>
-      <c r="AT70" s="39"/>
-    </row>
-    <row r="71" spans="3:46">
+      <c r="AT70" s="37"/>
+    </row>
+    <row r="71" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C71" s="20">
         <v>43</v>
       </c>
@@ -5782,9 +5775,9 @@
       <c r="AP71"/>
       <c r="AQ71"/>
       <c r="AR71"/>
-      <c r="AT71" s="39"/>
-    </row>
-    <row r="72" spans="3:46">
+      <c r="AT71" s="37"/>
+    </row>
+    <row r="72" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C72" s="20">
         <v>44</v>
       </c>
@@ -5824,9 +5817,9 @@
       <c r="AP72"/>
       <c r="AQ72"/>
       <c r="AR72"/>
-      <c r="AT72" s="39"/>
-    </row>
-    <row r="73" spans="3:46">
+      <c r="AT72" s="37"/>
+    </row>
+    <row r="73" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C73" s="20">
         <v>45</v>
       </c>
@@ -5866,9 +5859,9 @@
       <c r="AP73"/>
       <c r="AQ73"/>
       <c r="AR73"/>
-      <c r="AT73" s="39"/>
-    </row>
-    <row r="74" spans="3:46">
+      <c r="AT73" s="37"/>
+    </row>
+    <row r="74" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C74" s="20">
         <v>46</v>
       </c>
@@ -5908,9 +5901,9 @@
       <c r="AP74"/>
       <c r="AQ74"/>
       <c r="AR74"/>
-      <c r="AT74" s="39"/>
-    </row>
-    <row r="75" spans="3:46">
+      <c r="AT74" s="37"/>
+    </row>
+    <row r="75" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C75" s="20">
         <v>47</v>
       </c>
@@ -5950,9 +5943,9 @@
       <c r="AP75"/>
       <c r="AQ75"/>
       <c r="AR75"/>
-      <c r="AT75" s="39"/>
-    </row>
-    <row r="76" spans="3:46">
+      <c r="AT75" s="37"/>
+    </row>
+    <row r="76" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C76" s="20">
         <v>48</v>
       </c>
@@ -5992,9 +5985,9 @@
       <c r="AP76"/>
       <c r="AQ76"/>
       <c r="AR76"/>
-      <c r="AT76" s="39"/>
-    </row>
-    <row r="77" spans="3:46">
+      <c r="AT76" s="37"/>
+    </row>
+    <row r="77" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C77" s="20">
         <v>49</v>
       </c>
@@ -6034,9 +6027,9 @@
       <c r="AP77"/>
       <c r="AQ77"/>
       <c r="AR77"/>
-      <c r="AT77" s="39"/>
-    </row>
-    <row r="78" spans="3:46">
+      <c r="AT77" s="37"/>
+    </row>
+    <row r="78" spans="3:46" x14ac:dyDescent="0.2">
       <c r="C78" s="20">
         <v>50</v>
       </c>
@@ -6076,9 +6069,9 @@
       <c r="AP78"/>
       <c r="AQ78"/>
       <c r="AR78"/>
-      <c r="AT78" s="39"/>
-    </row>
-    <row r="79" spans="3:46">
+      <c r="AT78" s="37"/>
+    </row>
+    <row r="79" spans="3:46" x14ac:dyDescent="0.2">
       <c r="AJ79"/>
       <c r="AK79"/>
       <c r="AL79"/>
@@ -6088,9 +6081,9 @@
       <c r="AP79"/>
       <c r="AQ79"/>
       <c r="AR79"/>
-      <c r="AT79" s="39"/>
-    </row>
-    <row r="80" spans="3:46">
+      <c r="AT79" s="37"/>
+    </row>
+    <row r="80" spans="3:46" x14ac:dyDescent="0.2">
       <c r="AH80"/>
       <c r="AI80"/>
       <c r="AJ80"/>
@@ -6102,9 +6095,9 @@
       <c r="AP80"/>
       <c r="AQ80"/>
       <c r="AR80"/>
-      <c r="AT80" s="39"/>
-    </row>
-    <row r="81" spans="2:47">
+      <c r="AT80" s="37"/>
+    </row>
+    <row r="81" spans="2:47" x14ac:dyDescent="0.2">
       <c r="C81" s="26"/>
       <c r="D81" s="27"/>
       <c r="E81" s="27"/>
@@ -6128,26 +6121,26 @@
       <c r="AP81"/>
       <c r="AQ81"/>
       <c r="AR81"/>
-      <c r="AT81" s="39"/>
-    </row>
-    <row r="82" spans="2:47" ht="117" customHeight="1">
+      <c r="AT81" s="37"/>
+    </row>
+    <row r="82" spans="2:47" ht="117" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B82" s="25"/>
-      <c r="C82" s="37" t="s">
+      <c r="C82" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="D82" s="38"/>
-      <c r="E82" s="38"/>
-      <c r="F82" s="38"/>
-      <c r="G82" s="38"/>
-      <c r="H82" s="38"/>
-      <c r="O82" s="37" t="s">
+      <c r="D82" s="46"/>
+      <c r="E82" s="46"/>
+      <c r="F82" s="46"/>
+      <c r="G82" s="46"/>
+      <c r="H82" s="46"/>
+      <c r="O82" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="P82" s="38"/>
-      <c r="Q82" s="38"/>
-      <c r="R82" s="38"/>
-      <c r="S82" s="38"/>
-      <c r="T82" s="38"/>
+      <c r="P82" s="46"/>
+      <c r="Q82" s="46"/>
+      <c r="R82" s="46"/>
+      <c r="S82" s="46"/>
+      <c r="T82" s="46"/>
       <c r="AH82"/>
       <c r="AI82"/>
       <c r="AJ82"/>
@@ -6159,9 +6152,9 @@
       <c r="AP82"/>
       <c r="AQ82"/>
       <c r="AR82"/>
-      <c r="AT82" s="39"/>
-    </row>
-    <row r="83" spans="2:47">
+      <c r="AT82" s="37"/>
+    </row>
+    <row r="83" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AH83"/>
       <c r="AI83"/>
       <c r="AJ83"/>
@@ -6173,9 +6166,9 @@
       <c r="AP83"/>
       <c r="AQ83"/>
       <c r="AR83"/>
-      <c r="AT83" s="39"/>
-    </row>
-    <row r="84" spans="2:47">
+      <c r="AT83" s="37"/>
+    </row>
+    <row r="84" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AH84"/>
       <c r="AI84"/>
       <c r="AJ84"/>
@@ -6187,9 +6180,9 @@
       <c r="AP84"/>
       <c r="AQ84"/>
       <c r="AR84"/>
-      <c r="AT84" s="39"/>
-    </row>
-    <row r="85" spans="2:47">
+      <c r="AT84" s="37"/>
+    </row>
+    <row r="85" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AH85"/>
       <c r="AI85"/>
       <c r="AJ85"/>
@@ -6201,9 +6194,9 @@
       <c r="AP85"/>
       <c r="AQ85"/>
       <c r="AR85"/>
-      <c r="AT85" s="39"/>
-    </row>
-    <row r="86" spans="2:47">
+      <c r="AT85" s="37"/>
+    </row>
+    <row r="86" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AH86"/>
       <c r="AI86"/>
       <c r="AJ86"/>
@@ -6215,284 +6208,284 @@
       <c r="AP86"/>
       <c r="AQ86"/>
       <c r="AR86"/>
-      <c r="AT86" s="39"/>
-    </row>
-    <row r="87" spans="2:47">
+      <c r="AT86" s="37"/>
+    </row>
+    <row r="87" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AS87" s="2"/>
-      <c r="AT87" s="40"/>
-    </row>
-    <row r="88" spans="2:47">
+      <c r="AT87" s="38"/>
+    </row>
+    <row r="88" spans="2:47" x14ac:dyDescent="0.2">
       <c r="AS88" s="2"/>
-      <c r="AT88" s="40"/>
-    </row>
-    <row r="89" spans="2:47">
+      <c r="AT88" s="38"/>
+    </row>
+    <row r="89" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D89" s="2"/>
       <c r="E89" s="2"/>
       <c r="AS89" s="2"/>
-      <c r="AT89" s="40"/>
-    </row>
-    <row r="90" spans="2:47">
+      <c r="AT89" s="38"/>
+    </row>
+    <row r="90" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D90" s="2"/>
       <c r="E90" s="2"/>
-      <c r="AS90" s="43"/>
-      <c r="AT90" s="42"/>
-    </row>
-    <row r="91" spans="2:47">
+      <c r="AS90" s="40"/>
+      <c r="AT90" s="2"/>
+    </row>
+    <row r="91" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D91" s="2"/>
       <c r="E91" s="2"/>
-      <c r="AS91" s="43"/>
+      <c r="AS91" s="40"/>
       <c r="AU91"/>
     </row>
-    <row r="92" spans="2:47" s="41" customFormat="1" ht="17" thickBot="1">
-      <c r="AS92" s="44"/>
+    <row r="92" spans="2:47" s="39" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AS92" s="41"/>
       <c r="AT92"/>
       <c r="AU92"/>
     </row>
-    <row r="93" spans="2:47">
+    <row r="93" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D93" s="2"/>
       <c r="E93" s="2"/>
       <c r="AS93" s="2"/>
       <c r="AU93"/>
     </row>
-    <row r="94" spans="2:47">
+    <row r="94" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D94" s="2"/>
       <c r="E94" s="2"/>
     </row>
-    <row r="95" spans="2:47">
+    <row r="95" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D95" s="2"/>
       <c r="E95" s="2"/>
     </row>
-    <row r="96" spans="2:47">
+    <row r="96" spans="2:47" x14ac:dyDescent="0.2">
       <c r="D96" s="2"/>
       <c r="E96" s="2"/>
     </row>
-    <row r="97" spans="4:5" hidden="1">
+    <row r="97" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D97" s="2"/>
       <c r="E97" s="2"/>
     </row>
-    <row r="98" spans="4:5" hidden="1">
+    <row r="98" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D98" s="2"/>
       <c r="E98" s="2"/>
     </row>
-    <row r="99" spans="4:5" hidden="1">
+    <row r="99" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D99" s="2"/>
       <c r="E99" s="2"/>
     </row>
-    <row r="100" spans="4:5" hidden="1">
+    <row r="100" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D100" s="2"/>
       <c r="E100" s="2"/>
     </row>
-    <row r="101" spans="4:5" hidden="1">
+    <row r="101" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D101" s="2"/>
       <c r="E101" s="2"/>
     </row>
-    <row r="102" spans="4:5" hidden="1">
+    <row r="102" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D102" s="2"/>
       <c r="E102" s="2"/>
     </row>
-    <row r="103" spans="4:5" hidden="1">
+    <row r="103" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D103" s="2"/>
       <c r="E103" s="2"/>
     </row>
-    <row r="104" spans="4:5" hidden="1">
+    <row r="104" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D104" s="2"/>
       <c r="E104" s="2"/>
     </row>
-    <row r="105" spans="4:5" hidden="1">
+    <row r="105" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D105" s="2"/>
       <c r="E105" s="2"/>
     </row>
-    <row r="106" spans="4:5" hidden="1">
+    <row r="106" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D106" s="2"/>
       <c r="E106" s="2"/>
     </row>
-    <row r="107" spans="4:5" hidden="1">
+    <row r="107" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D107" s="2"/>
       <c r="E107" s="2"/>
     </row>
-    <row r="108" spans="4:5" hidden="1">
+    <row r="108" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D108" s="2"/>
       <c r="E108" s="2"/>
     </row>
-    <row r="109" spans="4:5" hidden="1">
+    <row r="109" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D109" s="2"/>
       <c r="E109" s="2"/>
     </row>
-    <row r="110" spans="4:5" hidden="1">
+    <row r="110" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D110" s="2"/>
       <c r="E110" s="2"/>
     </row>
-    <row r="111" spans="4:5" hidden="1">
+    <row r="111" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D111" s="2"/>
       <c r="E111" s="2"/>
     </row>
-    <row r="112" spans="4:5" hidden="1">
+    <row r="112" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D112" s="2"/>
       <c r="E112" s="2"/>
     </row>
-    <row r="113" spans="4:5" hidden="1">
+    <row r="113" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D113" s="2"/>
       <c r="E113" s="2"/>
     </row>
-    <row r="114" spans="4:5" hidden="1">
+    <row r="114" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D114" s="2"/>
       <c r="E114" s="2"/>
     </row>
-    <row r="115" spans="4:5" hidden="1">
+    <row r="115" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D115" s="2"/>
       <c r="E115" s="2"/>
     </row>
-    <row r="116" spans="4:5" hidden="1">
+    <row r="116" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D116" s="2"/>
       <c r="E116" s="2"/>
     </row>
-    <row r="117" spans="4:5" hidden="1">
+    <row r="117" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D117" s="2"/>
       <c r="E117" s="2"/>
     </row>
-    <row r="118" spans="4:5" hidden="1">
+    <row r="118" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D118" s="2"/>
       <c r="E118" s="2"/>
     </row>
-    <row r="119" spans="4:5" hidden="1">
+    <row r="119" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D119" s="2"/>
       <c r="E119" s="2"/>
     </row>
-    <row r="120" spans="4:5" hidden="1">
+    <row r="120" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D120" s="2"/>
       <c r="E120" s="2"/>
     </row>
-    <row r="121" spans="4:5" hidden="1">
+    <row r="121" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D121" s="2"/>
       <c r="E121" s="2"/>
     </row>
-    <row r="122" spans="4:5" hidden="1">
+    <row r="122" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D122" s="2"/>
       <c r="E122" s="2"/>
     </row>
-    <row r="123" spans="4:5" hidden="1">
+    <row r="123" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D123" s="2"/>
       <c r="E123" s="2"/>
     </row>
-    <row r="124" spans="4:5" hidden="1">
+    <row r="124" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D124" s="2"/>
       <c r="E124" s="2"/>
     </row>
-    <row r="125" spans="4:5" hidden="1">
+    <row r="125" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D125" s="2"/>
       <c r="E125" s="2"/>
     </row>
-    <row r="126" spans="4:5" hidden="1">
+    <row r="126" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D126" s="2"/>
       <c r="E126" s="2"/>
     </row>
-    <row r="127" spans="4:5" hidden="1">
+    <row r="127" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D127" s="2"/>
       <c r="E127" s="2"/>
     </row>
-    <row r="128" spans="4:5" hidden="1">
+    <row r="128" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D128" s="2"/>
       <c r="E128" s="2"/>
     </row>
-    <row r="129" spans="4:5" hidden="1">
+    <row r="129" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D129" s="2"/>
       <c r="E129" s="2"/>
     </row>
-    <row r="130" spans="4:5" hidden="1">
+    <row r="130" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D130" s="2"/>
       <c r="E130" s="2"/>
     </row>
-    <row r="131" spans="4:5" hidden="1">
+    <row r="131" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D131" s="2"/>
       <c r="E131" s="2"/>
     </row>
-    <row r="132" spans="4:5" hidden="1">
+    <row r="132" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D132" s="2"/>
       <c r="E132" s="2"/>
     </row>
-    <row r="133" spans="4:5" hidden="1">
+    <row r="133" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D133" s="2"/>
       <c r="E133" s="2"/>
     </row>
-    <row r="134" spans="4:5" hidden="1">
+    <row r="134" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D134" s="2"/>
       <c r="E134" s="2"/>
     </row>
-    <row r="135" spans="4:5" hidden="1">
+    <row r="135" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D135" s="2"/>
       <c r="E135" s="2"/>
     </row>
-    <row r="136" spans="4:5" hidden="1">
+    <row r="136" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D136" s="2"/>
       <c r="E136" s="2"/>
     </row>
-    <row r="137" spans="4:5" hidden="1">
+    <row r="137" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D137" s="2"/>
       <c r="E137" s="2"/>
     </row>
-    <row r="138" spans="4:5" hidden="1">
+    <row r="138" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D138" s="2"/>
       <c r="E138" s="2"/>
     </row>
-    <row r="139" spans="4:5" hidden="1">
+    <row r="139" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D139" s="2"/>
       <c r="E139" s="2"/>
     </row>
-    <row r="140" spans="4:5" hidden="1">
+    <row r="140" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D140" s="2"/>
       <c r="E140" s="2"/>
     </row>
-    <row r="141" spans="4:5" hidden="1">
+    <row r="141" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D141" s="2"/>
       <c r="E141" s="2"/>
     </row>
-    <row r="142" spans="4:5" hidden="1">
+    <row r="142" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D142" s="2"/>
       <c r="E142" s="2"/>
     </row>
-    <row r="143" spans="4:5" hidden="1">
+    <row r="143" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D143" s="2"/>
       <c r="E143" s="2"/>
     </row>
-    <row r="144" spans="4:5" hidden="1">
+    <row r="144" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D144" s="2"/>
       <c r="E144" s="2"/>
     </row>
-    <row r="145" spans="4:5" hidden="1">
+    <row r="145" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D145" s="2"/>
       <c r="E145" s="2"/>
     </row>
-    <row r="146" spans="4:5" hidden="1">
+    <row r="146" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D146" s="2"/>
       <c r="E146" s="2"/>
     </row>
-    <row r="147" spans="4:5" hidden="1">
+    <row r="147" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D147" s="2"/>
       <c r="E147" s="2"/>
     </row>
-    <row r="148" spans="4:5" hidden="1">
+    <row r="148" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D148" s="2"/>
       <c r="E148" s="2"/>
     </row>
-    <row r="149" spans="4:5" hidden="1">
+    <row r="149" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D149" s="2"/>
       <c r="E149" s="2"/>
     </row>
-    <row r="150" spans="4:5" hidden="1">
+    <row r="150" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D150" s="2"/>
       <c r="E150" s="2"/>
     </row>
-    <row r="151" spans="4:5" hidden="1">
+    <row r="151" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D151" s="2"/>
       <c r="E151" s="2"/>
     </row>
-    <row r="152" spans="4:5" hidden="1">
+    <row r="152" spans="4:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D152" s="2"/>
       <c r="E152" s="2"/>
     </row>
-    <row r="153" spans="4:5"/>
-    <row r="154" spans="4:5"/>
-    <row r="155" spans="4:5"/>
+    <row r="153" spans="4:5" x14ac:dyDescent="0.2"/>
+    <row r="154" spans="4:5" x14ac:dyDescent="0.2"/>
+    <row r="155" spans="4:5" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="C82:H82"/>

</xml_diff>